<commit_message>
Updated usb2p0 testcases file in docs
</commit_message>
<xml_diff>
--- a/USB2p0_VIP/Docs/USB2p0_Testcases.xlsx
+++ b/USB2p0_VIP/Docs/USB2p0_Testcases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30117"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30128"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://siliciomtech-my.sharepoint.com/personal/shruti_p_siliciom_com/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A0776031-CF79-4A05-B7AC-91205D63073C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E9BFB8DC-C854-4C29-82E0-EC29D52318A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="USB 2p0 Testplan" sheetId="2" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1000" uniqueCount="616">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1040" uniqueCount="650">
   <si>
     <t>S.No</t>
   </si>
@@ -2936,7 +2936,10 @@
     <t>Assertion Property</t>
   </si>
   <si>
-    <t>usb2p0_dp_dm_comp</t>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>usb2p0_p_dp_dm_not_both_high</t>
   </si>
   <si>
     <t>The dp_dm_complement assertion is implemented to verify that the USB differential signals Dp and Dm are always complementary during operation.
@@ -2944,14 +2947,17 @@
 This ensures correct differential signaling behavior required for valid USB communication</t>
   </si>
   <si>
-    <t xml:space="preserve">property p_dp_dm_complement;
-    @(posedge phy_clk)
-    (Dp !== Dm);
+    <t xml:space="preserve">property p_dp_dm_not_both_high;
+   @(posedge clk) disable iff (reset)
+   not (dp === 1'b1 &amp;&amp; dm === 1'b1);
 endproperty
 </t>
   </si>
   <si>
-    <t>usb2p0_rxvalid_rxactive</t>
+    <t>29/05/2026</t>
+  </si>
+  <si>
+    <t>usb2p0_p_rxvalid_with_rxactive</t>
   </si>
   <si>
     <t>The rxvalid_with_rxactive assertion is implemented to verify that utmi_rxactive is asserted whenever utmi_rxvalid is high.
@@ -2967,7 +2973,7 @@
 </t>
   </si>
   <si>
-    <t>usb2p0_txvalid_txready</t>
+    <t>usb2p0_p_txvalid_txready_handshake</t>
   </si>
   <si>
     <t>The txvalid_txready_handshake assertion is implemented to verify the UTMI transmit handshake behavior between utmi_txvalid and utmi_txready.
@@ -2977,13 +2983,13 @@
   </si>
   <si>
     <t xml:space="preserve">property p_txvalid_txready_handshake;
-    @(posedge utmi_clk)
+ @(posedge utmi_clk)
     utmi_txvalid |-&gt; ##[0:5] utmi_txready;
 endproperty
 </t>
   </si>
   <si>
-    <t>usb2p0_txvalid_txdata</t>
+    <t>usb2p0_p_txdata_not_unknown</t>
   </si>
   <si>
     <t>The txdata_not_unknown assertion is implemented to verify that transmitted UTMI data does not contain unknown (X or Z) values during valid transmission.
@@ -2993,13 +2999,13 @@
   </si>
   <si>
     <t xml:space="preserve">property p_txdata_not_unknown;
-    @(posedge utmi_clk)
+   @(posedge utmi_clk)
     utmi_txvalid |-&gt; (!$isunknown(utmi_txdata));
 endproperty
 </t>
   </si>
   <si>
-    <t>usb2p0_rxvalid_rxdata</t>
+    <t>usb2p0_p_rxdata_not_unknown</t>
   </si>
   <si>
     <t>The rxdata_not_unknown assertion is implemented to verify that received UTMI data does not contain unknown (X or Z) values during valid reception.
@@ -3009,24 +3015,8 @@
   </si>
   <si>
     <t xml:space="preserve">property p_rxdata_not_unknown;
-    @(posedge utmi_clk)
+ @(posedge utmi_clk)
     utmi_rxvalid |-&gt; (!$isunknown(utmi_rxdata));
-endproperty
-</t>
-  </si>
-  <si>
-    <t>usb2p0_linestate</t>
-  </si>
-  <si>
-    <t>The p_linestate_known assertion is implemented to verify that the utmi_linestate signal never contains unknown (X or Z) values.
-It checks on every positive edge of utmi_clk that the line state information remains valid and deterministic.
-This ensures correct USB PHY line state monitoring and signaling behavior during operation.
-The assertion helps detect invalid or uninitialized UTMI line state conditions during simulation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">property p_linestate_known;
-    @(posedge utmi_clk)
-    !$isunknown(utmi_linestate);
 endproperty
 </t>
   </si>
@@ -3041,8 +3031,8 @@
   </si>
   <si>
     <t xml:space="preserve">property p_ls_fs_mode_check;
-    @(posedge utmi_clk)
-    (!utmi_txvalidh &amp;&amp; !utmi_rxvalidh) |-&gt; (utmi_word_if == 1'b0);
+@(posedge utmi_clk)
+    (!utmi_txvalidh &amp;&amp; !utmi_rxvalidh &amp;&amp; utmi_txvalid &amp;&amp; utmi_rxvalid) |-&gt; (utmi_word_if == 1'b0);
 endproperty
 </t>
   </si>
@@ -3060,38 +3050,148 @@
 </t>
   </si>
   <si>
-    <t>usb2p0_vbus</t>
-  </si>
-  <si>
-    <t>The vbus_valid assertion is implemented to verify correct USB OTG VBUS validity signaling behavior.
-It checks that whenever utmiotg_vbusvalid is asserted, the utmisrp_bvalid signal is also asserted.
-This ensures proper detection and handling of valid VBUS conditions during OTG operation.
-The assertion helps detect invalid power signaling and OTG protocol violations during simulation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">property p_vbus_valid;
-    @(posedge utmi_clk)
-    utmiotg_vbusvalid |-&gt; utmisrp_bvalid;
+    <t>usb2p0_p_pid_check</t>
+  </si>
+  <si>
+    <t>Verifies the USB PID format whenever a valid PID is detected. 
+The assertion checks that the upper 4 bits of the PID field are the bitwise complement of the lower 4 bits, as required by the USB 2.0 specification.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">property p_pid_check;
+  @(posedge clk) disable iff (reset)
+  $rose(pid_valid) |-&gt; (pid_byte[7:4] == ~pid_byte[3:0]);
 endproperty
 </t>
   </si>
   <si>
-    <t>usb2p0_dp_dm</t>
-  </si>
-  <si>
-    <t>The dp_dm_pulldown assertion is implemented to verify that both utmiotg_dppulldown and utmiotg_dmpulldown are not asserted simultaneously.
-It checks on every positive edge of utmi_clk to prevent invalid USB OTG pulldown control conditions.
-This ensures proper USB line control and OTG signaling behavior during operation.
-The assertion helps detect incorrect PHY pulldown configuration and protocol violations during simulation.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">property p_dp_dm_pulldown;
-    @(posedge utmi_clk)
-    !(utmiotg_dppulldown &amp;&amp; utmiotg_dmpulldown);
+    <t>usb2p0_p_pid_legal</t>
+  </si>
+  <si>
+    <t>Verifies that every received PID corresponds to a supported and legal USB packet identifier. 
+The assertion checks the PID type field (lower nibble) against a predefined list of valid USB PIDs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">property p_pid_legal;
+  @(posedge utmi_clk) disable iff (reset)
+  $rose(pid_valid) |-&gt;
+    pid_byte[3:0] inside {
+      4'hE, // OUT
+      4'h6, // IN
+      4'h2, // SETUP
+      4'hC, // DATA0
+      4'h4, // DATA1
+      4'hD, // ACK
+      4'h5, // NAK
+      4'h1 // STALL
+    };
 endproperty
 </t>
   </si>
   <si>
+    <t>usb2p0_p_in_transaction_order</t>
+  </si>
+  <si>
+    <t>Verifies the correct packet sequence of a USB IN transaction.
+ After the host transmits an IN token, the device must respond with a DATA1 packet, followed by an ACK handshake from the host.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">property p_in_transaction_order;
+  @(posedge utmi_clk) disable iff (reset)
+    (pid_valid &amp;&amp; pid_byte[3:0] == 4'h6) |-&gt;
+    ##[1:128] (device_pid_valid &amp;&amp; device_pid_byte[3:0] == 4'h4)
+    ##[1:128] (pid_valid &amp;&amp; pid_byte[3:0] == 4'hd);
+endproperty
+</t>
+  </si>
+  <si>
+    <t>usb2p0_p_out_transaction_order</t>
+  </si>
+  <si>
+    <t>Verifies the correct packet sequence of a USB OUT transaction. 
+After the host transmits an OUT token, the host must send a DATA1 packet, and the device must respond with an ACK handshake.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">property p_out_transaction_order;
+  @(posedge utmi_clk) disable iff (reset)
+    $rose(txvalid &amp;&amp; pid_byte[3:0]==4'he) |-&gt;
+    ##[1:256] (pid_valid &amp;&amp; pid_byte[3:0]==4'h4)
+    ##[1:256] (device_pid_valid &amp;&amp; device_pid_byte[3:0]==4'hd);
+endproperty
+</t>
+  </si>
+  <si>
+    <t>usb2p0_p_setup_uses_data0</t>
+  </si>
+  <si>
+    <t>Verifies that every USB SETUP transaction uses a DATA0 packet as the data stage PID.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">property p_setup_uses_data0;
+  @(posedge utmi_clk) disable iff (reset)
+    $rose(txvalid &amp;&amp; pid_byte[3:0] == 4'h2) |-&gt;
+    ##[1:256] (data_valid || pid_byte[3:0] == 4'hc)  // DATA0
+    ##[1:256] (device_pid_valid &amp;&amp; device_pid_byte[3:0]==4'hd);
+endproperty
+</t>
+  </si>
+  <si>
+    <t>usb2p0_p_inter_packet_gap</t>
+  </si>
+  <si>
+    <t>Verifies that a minimum Inter-Packet Gap (IPG) is maintained between the end of one packet and the start of the next packet.
+ The assertion checks that after a packet transmission completes (pkt_active deasserts), the bus remains idle for at least 10 clock cycles before another packet transmission begins.</t>
+  </si>
+  <si>
+    <t>property p_inter_packet_gap;
+  @(posedge clk) disable iff (reset)
+  $fell(pkt_active) |-&gt; ##[10:$] $rose(pkt_active);  
+endproperty
+a_inter_packet_gap: assert property (p_inter_packet_gap)
+  else $warning("IPG: next_packet_started_before_2-bit_gap_elapsed");</t>
+  </si>
+  <si>
+    <t>usb2p0_p_no_handshake_after_token_direct</t>
+  </si>
+  <si>
+    <t>Verifies that a handshake packet is not generated immediately after a token packet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">property p_no_handshake_after_token_direct;
+  @(posedge clk) disable iff (reset)
+  $rose(token_valid) |-&gt; !handshake_valid[*1:5];
+endproperty
+</t>
+  </si>
+  <si>
+    <t>usb2p0_p_linestate_known</t>
+  </si>
+  <si>
+    <t>Verifies that the UTMI utmi_linestate signal becomes a known and valid value within 1 to 10 UTMI clock cycles after utmiotg_vbusvalid is asserted. This ensures that once valid VBUS power is detected, the PHY correctly reports the USB line state and does not drive unknown (X) or high-impedance (Z) values on the utmi_linestate signal.</t>
+  </si>
+  <si>
+    <t>property p_linestate_known;
+   @(posedge utmi_clk)
+   $rose(utmiotg_vbusvalid) |-&gt; ##[1:10] (!$isunknown(utmi_linestate));
+endproperty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      4/6/206</t>
+  </si>
+  <si>
+    <t>usb2p0_p_vbus_valid</t>
+  </si>
+  <si>
+    <t>Verifies that the Session Request Protocol (SRP) valid indication (utmisrp_bvalid) is asserted within 1 to 10 UTMI clock cycles after the VBUS valid signal (utmiotg_vbusvalid) is asserted. 
+This ensures proper detection and propagation of VBUS validity to the UTMI OTG status signals.</t>
+  </si>
+  <si>
+    <t>property p_vbus_valid;
+   @(posedge utmi_clk)
+   disable iff(reset)
+   $rose(utmiotg_vbusvalid) |-&gt; ##[1:10] utmisrp_bvalid;
+endproperty</t>
+  </si>
+  <si>
     <t>Chandan</t>
   </si>
   <si>
@@ -3398,7 +3498,7 @@
     <t xml:space="preserve">  covergroup usb_pid_cg;</t>
   </si>
   <si>
-    <t>USB_PID_CP :coverpoint pidsample_host_tx</t>
+    <t xml:space="preserve">USB_PID_CP </t>
   </si>
   <si>
     <t>The USB_PID_CP coverpoint is implemented to verify the coverage of different USB2.0 PID packets transmitted through the Host TX interface.
@@ -3419,7 +3519,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve"> ADDR: coverpoint usb_seq_item.addr</t>
+    <t xml:space="preserve"> USB_ADDR_CP</t>
   </si>
   <si>
     <t>The ADDR coverpoint is implemented to verify the USB default device address behavior during enumeration. 
@@ -3435,7 +3535,7 @@
                                                                                                        </t>
   </si>
   <si>
-    <t>ENDPOINT : coverpoint usb_seq_item.endp</t>
+    <t>USB_ENDPOINT_CP</t>
   </si>
   <si>
     <t>The ENDPOINT coverpoint is implemented to verify that all supported USB endpoints are exercised during simulation.
@@ -3459,7 +3559,7 @@
                                                                                           </t>
   </si>
   <si>
-    <t xml:space="preserve"> BREQUEST: coverpoint usb_seq_item.bRequest</t>
+    <t xml:space="preserve"> USB_BREQUEST_CP</t>
   </si>
   <si>
     <t>The BREQUEST coverpoint is implemented to verify that all valid USB standard device requests are exercised during simulation.
@@ -3486,7 +3586,7 @@
 </t>
   </si>
   <si>
-    <t>BMREQUESTTYPE : coverpoint  usb_seq_item.bmRequestType</t>
+    <t>USB_BMREQUESTTYPE_CP</t>
   </si>
   <si>
     <t>The BMREQUESTTYPE coverpoint is implemented to verify valid USB request type fields during control transfer transactions.
@@ -3505,7 +3605,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve"> WVALUE : coverpoint usb_seq_item.wValue</t>
+    <t xml:space="preserve"> USB_WVALUE_CP</t>
   </si>
   <si>
     <t>The WVALUE coverpoint is implemented to verify important USB wValue field values during control transfer transactions.
@@ -3522,7 +3622,7 @@
                                                         }                                                                                                                                 </t>
   </si>
   <si>
-    <t xml:space="preserve"> WINDEX : coverpoint usb_seq_item.wIndex</t>
+    <t xml:space="preserve"> USB_WINDEX _CP</t>
   </si>
   <si>
     <t>The WINDEX coverpoint is implemented to verify important USB wIndex field values during control transfer transactions.
@@ -3539,7 +3639,7 @@
                                                    ignore_bins  = {[0:65535]} with (!(item inside {16'h0000,16'h0001,16'h0081}));       </t>
   </si>
   <si>
-    <t xml:space="preserve"> WLENGTH : coverpoint  usb_seq_item.wLength</t>
+    <t>USB_ WLENGTH_CP</t>
   </si>
   <si>
     <t>The WLENGTH coverpoint is implemented to verify important USB wLength field values during control transfer transactions.
@@ -3558,7 +3658,7 @@
                                                                                                  </t>
   </si>
   <si>
-    <t>BLENGTH : coverpoint usb_seq_item.blength</t>
+    <t>USB_BLENGTH_CP</t>
   </si>
   <si>
     <t>The BLENGTH coverpoint is implemented to verify the USB descriptor length field during descriptor-related transactions.
@@ -3575,7 +3675,7 @@
  </t>
   </si>
   <si>
-    <t>DESC_TYPE : coverpoint usb_seq_item.bdescriptors_type</t>
+    <t>USB_DESC_TYPE_CP</t>
   </si>
   <si>
     <t>The DESC_TYPE coverpoint is implemented to verify the USB descriptor type field during descriptor request transactions.
@@ -3592,7 +3692,7 @@
 </t>
   </si>
   <si>
-    <t>BCD_USB : coverpoint usb_seq_item.bcd_usb</t>
+    <t>USB_BCD_USB_CP</t>
   </si>
   <si>
     <t>The lBCD_USB coverpoint is implemented to verify the USB specification version field in the device descriptor.
@@ -3609,7 +3709,7 @@
                                                                                                                                       </t>
   </si>
   <si>
-    <t>DEVICE_CLASS : coverpoint usb_seq_item.bDevice_class</t>
+    <t>USB_DEVICE_CLASS_CP</t>
   </si>
   <si>
     <t>The DEVICE_CLASS coverpoint is implemented to verify the USB device class field in the device descriptor.
@@ -3625,7 +3725,7 @@
                                                                                                          }</t>
   </si>
   <si>
-    <t xml:space="preserve">DEVICE_SUBCLASS : coverpoint usb_seq_item.bDevice_subclass </t>
+    <t xml:space="preserve">USB_DEVICE_SUBCLASS_CP </t>
   </si>
   <si>
     <t>The DEVICE_SUBCLASS coverpoint is implemented to verify the USB device subclass field in the device descriptor.
@@ -3640,7 +3740,7 @@
                                                                                                        }                                                                                              </t>
   </si>
   <si>
-    <t xml:space="preserve">DEVICE_PROTOCOL : coverpoint usb_seq_item.bDevice_protocol
+    <t xml:space="preserve">USB_DEVICE_PROTOCOL_CP
 </t>
   </si>
   <si>
@@ -3656,7 +3756,7 @@
                                                                                                       }</t>
   </si>
   <si>
-    <t xml:space="preserve">          MAX_PACKET : coverpoint usb_seq_item.bMax_packetsize 
+    <t xml:space="preserve">          USB_MAX_PACKET_CP
 </t>
   </si>
   <si>
@@ -3673,7 +3773,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">VENDOR_ID : coverpoint usb_seq_item.idvendor 
+    <t xml:space="preserve">USB_VENDOR_ID_CP
 </t>
   </si>
   <si>
@@ -3689,7 +3789,7 @@
                                                                                                   }</t>
   </si>
   <si>
-    <t xml:space="preserve">PRODUCT_ID : coverpoint usb_seq_item.idproduct 
+    <t xml:space="preserve">USB_PRODUCT_ID_CP 
 </t>
   </si>
   <si>
@@ -3706,7 +3806,7 @@
  </t>
   </si>
   <si>
-    <t xml:space="preserve">DEVICE_BCD : coverpoint usb_seq_item.bcdDevice 
+    <t xml:space="preserve">USB_DEVICE_BCD_CP 
 </t>
   </si>
   <si>
@@ -3721,7 +3821,7 @@
                                                          ignore_bins  = {[0:65535]} with (item != 16'h0126);                                                                                                 }</t>
   </si>
   <si>
-    <t xml:space="preserve">  MANUF_STR : coverpoint usb_seq_item.imanufacture 
+    <t xml:space="preserve">  USB_MANUF_STR_CP 
 </t>
   </si>
   <si>
@@ -3736,7 +3836,7 @@
                                                       }</t>
   </si>
   <si>
-    <t xml:space="preserve">PROD_STR : coverpoint usb_seq_item.iproduct 
+    <t xml:space="preserve">USB_PROD_STR_CP 
 </t>
   </si>
   <si>
@@ -3753,7 +3853,7 @@
  </t>
   </si>
   <si>
-    <t xml:space="preserve">SERIAL_STR : coverpoint usb_seq_item.iserial_number </t>
+    <t xml:space="preserve">USB_SERIAL_STR_CP </t>
   </si>
   <si>
     <t>The SERIAL_STR coverpoint is implemented to verify the serial number string index field in the USB device descriptor.
@@ -3768,7 +3868,7 @@
                                                                                                   }</t>
   </si>
   <si>
-    <t xml:space="preserve">NUM_CONFIG : coverpoint usb_seq_item.bNum_configuration 
+    <t xml:space="preserve">USB_NUM_CONFIG_CP 
 </t>
   </si>
   <si>
@@ -3784,7 +3884,7 @@
                                                                                                         }</t>
   </si>
   <si>
-    <t xml:space="preserve">  TX_VALID  : coverpoint usb_seq_item.tx_valid;
+    <t xml:space="preserve">  USB_TX_VALID_CP 
 </t>
   </si>
   <si>
@@ -3793,7 +3893,11 @@
 The coverage helps confirm correct UTMI transmit interface behavior during packet transmission.</t>
   </si>
   <si>
-    <t xml:space="preserve">   TX_VALIDH  : coverpoint usb_seq_item.tx_validh;
+    <t xml:space="preserve">  TX_VALID  : coverpoint usb_seq_item.tx_valid;
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   USB_TX_VALIDH_CP
 </t>
   </si>
   <si>
@@ -3802,8 +3906,11 @@
 The coverage helps confirm correct high-speed USB transmit operation handling.</t>
   </si>
   <si>
-    <t xml:space="preserve">  RX_VALID  : coverpoint usb_seq_item.rx_valid;
+    <t xml:space="preserve">   TX_VALIDH  : coverpoint usb_seq_item.tx_validh;
 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  USB_RX_VALID_CP</t>
   </si>
   <si>
     <t>The RX_VALID coverpoint is implemented to verify receive valid signaling during USB packet reception.
@@ -3811,7 +3918,11 @@
 The coverage helps confirm correct UTMI receive interface behavior during packet reception.</t>
   </si>
   <si>
-    <t xml:space="preserve">   RX_VALIDH : coverpoint usb_seq_item.rx_validh;
+    <t xml:space="preserve">  RX_VALID  : coverpoint usb_seq_item.rx_valid;
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   USB_RX_VALIDH_CP
 </t>
   </si>
   <si>
@@ -3820,7 +3931,11 @@
 The coverage helps confirm correct high-speed USB receive operation handling.</t>
   </si>
   <si>
-    <t xml:space="preserve">    WORD_IF   : coverpoint  usb_seq_item.word_if;</t>
+    <t xml:space="preserve">   RX_VALIDH : coverpoint usb_seq_item.rx_validh;
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    USB_WORD_IF_CP  </t>
   </si>
   <si>
     <t>The WORD_IF coverpoint is implemented to verify word interface mode operation in the UTMI interface.
@@ -3828,7 +3943,10 @@
 The coverage helps confirm correct UTMI interface configuration handling.</t>
   </si>
   <si>
-    <t xml:space="preserve">OP_MODE : coverpoint usb_seq_item.op_mode 
+    <t xml:space="preserve">    WORD_IF   : coverpoint  usb_seq_item.word_if;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB_OP_MODE_CP 
 </t>
   </si>
   <si>
@@ -3843,7 +3961,7 @@
                                                    }</t>
   </si>
   <si>
-    <t xml:space="preserve">        TERM_SELECT : coverpoint usb_seq_item.term_select;
+    <t xml:space="preserve">USB_TERM_SELECT_CP
 </t>
   </si>
   <si>
@@ -3852,7 +3970,11 @@
 The coverage helps confirm correct PHY termination behavior handling.</t>
   </si>
   <si>
-    <t xml:space="preserve">        XCVR_SELECT : coverpoint usb_seq_item.xcvr_select;
+    <t xml:space="preserve">        TERM_SELECT : coverpoint usb_seq_item.term_select;
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> USB_XCVR_SELECT_CP 
 </t>
   </si>
   <si>
@@ -3861,7 +3983,11 @@
 The coverage helps confirm correct PHY transceiver configuration handling.</t>
   </si>
   <si>
-    <t xml:space="preserve">        SUSPEND_N : coverpoint usb_seq_item.suspend_n;
+    <t xml:space="preserve">        XCVR_SELECT : coverpoint usb_seq_item.xcvr_select;
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB_SUSPEND_N_CP 
 </t>
   </si>
   <si>
@@ -3870,7 +3996,11 @@
 The coverage helps confirm correct USB power management behavior.</t>
   </si>
   <si>
-    <t xml:space="preserve">       FSLS_SERIALMODE : coverpoint usb_seq_item.fsls_serialmode;
+    <t xml:space="preserve">        SUSPEND_N : coverpoint usb_seq_item.suspend_n;
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> USB_FSLS_SERIALMODE_CP 
 </t>
   </si>
   <si>
@@ -3879,7 +4009,11 @@
 The coverage helps confirm correct FS/LS serial communication handling.</t>
   </si>
   <si>
-    <t xml:space="preserve">       FSLS_LOW_POWER : coverpoint usb_seq_item.fsls_low_power;
+    <t xml:space="preserve">       FSLS_SERIALMODE : coverpoint usb_seq_item.fsls_serialmode;
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> USB_FSLS_LOW_POWER_CP
 </t>
   </si>
   <si>
@@ -3888,7 +4022,11 @@
 The coverage helps confirm correct USB low-power mode handling.</t>
   </si>
   <si>
-    <t xml:space="preserve">       OTG_DPPULLDOWN : coverpoint usb_seq_item.otg_dppulldown;
+    <t xml:space="preserve">       FSLS_LOW_POWER : coverpoint usb_seq_item.fsls_low_power;
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB_OTG_DPPULLDOWN_CP 
 </t>
   </si>
   <si>
@@ -3897,7 +4035,11 @@
 The coverage helps confirm correct OTG DP pulldown handling.</t>
   </si>
   <si>
-    <t xml:space="preserve">       OTG_DMPULLDOWN : coverpoint usb_seq_item.otg_dmpulldown;
+    <t xml:space="preserve">       OTG_DPPULLDOWN : coverpoint usb_seq_item.otg_dppulldown;
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USB_OTG_DMPULLDOWN_CP 
 </t>
   </si>
   <si>
@@ -3906,12 +4048,19 @@
 The coverage helps confirm correct OTG DM pulldown handling.</t>
   </si>
   <si>
-    <t xml:space="preserve">       UTMI_VALID_CROSS : cross TX_VALID, RX_VALID;</t>
+    <t xml:space="preserve">       OTG_DMPULLDOWN : coverpoint usb_seq_item.otg_dmpulldown;
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> USB_UTMI_VALID_CROSS_CP</t>
   </si>
   <si>
     <t>The UTMI_VALID_CROSS cross coverage is implemented to verify the interaction between transmit valid and receive valid signaling.
 It ensures that both TX and RX valid conditions are exercised together during simulation.
 The coverage helps confirm correct UTMI transmit and receive activity combinations.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">       UTMI_VALID_CROSS : cross TX_VALID, RX_VALID;</t>
   </si>
 </sst>
 </file>
@@ -4009,7 +4158,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4040,8 +4189,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -4145,11 +4300,33 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -4256,14 +4433,22 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -4277,6 +4462,27 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10117,7 +10323,7 @@
       <c r="A2" s="22">
         <v>1</v>
       </c>
-      <c r="B2" s="52" t="s">
+      <c r="B2" s="62" t="s">
         <v>9</v>
       </c>
       <c r="C2" s="23" t="s">
@@ -10146,7 +10352,7 @@
       <c r="A3" s="22">
         <v>2</v>
       </c>
-      <c r="B3" s="52"/>
+      <c r="B3" s="62"/>
       <c r="C3" s="22" t="s">
         <v>16</v>
       </c>
@@ -10173,7 +10379,7 @@
       <c r="A4" s="22">
         <v>3</v>
       </c>
-      <c r="B4" s="52" t="s">
+      <c r="B4" s="62" t="s">
         <v>22</v>
       </c>
       <c r="C4" s="22" t="s">
@@ -10202,7 +10408,7 @@
       <c r="A5" s="22">
         <v>4</v>
       </c>
-      <c r="B5" s="52"/>
+      <c r="B5" s="62"/>
       <c r="C5" s="22" t="s">
         <v>28</v>
       </c>
@@ -10229,7 +10435,7 @@
       <c r="A6" s="22">
         <v>5</v>
       </c>
-      <c r="B6" s="52"/>
+      <c r="B6" s="62"/>
       <c r="C6" s="22" t="s">
         <v>32</v>
       </c>
@@ -10256,10 +10462,10 @@
       <c r="A7" s="22">
         <v>6</v>
       </c>
-      <c r="B7" s="52" t="s">
+      <c r="B7" s="62" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="50" t="s">
+      <c r="C7" s="61" t="s">
         <v>38</v>
       </c>
       <c r="D7" s="22" t="s">
@@ -10285,8 +10491,8 @@
       <c r="A8" s="22">
         <v>7</v>
       </c>
-      <c r="B8" s="52"/>
-      <c r="C8" s="50"/>
+      <c r="B8" s="62"/>
+      <c r="C8" s="61"/>
       <c r="D8" s="22" t="s">
         <v>42</v>
       </c>
@@ -10310,8 +10516,8 @@
       <c r="A9" s="22">
         <v>8</v>
       </c>
-      <c r="B9" s="52"/>
-      <c r="C9" s="50"/>
+      <c r="B9" s="62"/>
+      <c r="C9" s="61"/>
       <c r="D9" s="22" t="s">
         <v>46</v>
       </c>
@@ -10335,8 +10541,8 @@
       <c r="A10" s="22">
         <v>9</v>
       </c>
-      <c r="B10" s="52"/>
-      <c r="C10" s="50" t="s">
+      <c r="B10" s="62"/>
+      <c r="C10" s="61" t="s">
         <v>49</v>
       </c>
       <c r="D10" s="22" t="s">
@@ -10362,8 +10568,8 @@
       <c r="A11" s="22">
         <v>10</v>
       </c>
-      <c r="B11" s="52"/>
-      <c r="C11" s="50"/>
+      <c r="B11" s="62"/>
+      <c r="C11" s="61"/>
       <c r="D11" s="22" t="s">
         <v>53</v>
       </c>
@@ -10387,8 +10593,8 @@
       <c r="A12" s="22">
         <v>11</v>
       </c>
-      <c r="B12" s="52"/>
-      <c r="C12" s="50"/>
+      <c r="B12" s="62"/>
+      <c r="C12" s="61"/>
       <c r="D12" s="22" t="s">
         <v>55</v>
       </c>
@@ -10412,8 +10618,8 @@
       <c r="A13" s="22">
         <v>12</v>
       </c>
-      <c r="B13" s="52"/>
-      <c r="C13" s="50" t="s">
+      <c r="B13" s="62"/>
+      <c r="C13" s="61" t="s">
         <v>58</v>
       </c>
       <c r="D13" s="22" t="s">
@@ -10439,8 +10645,8 @@
       <c r="A14" s="22">
         <v>13</v>
       </c>
-      <c r="B14" s="52"/>
-      <c r="C14" s="50"/>
+      <c r="B14" s="62"/>
+      <c r="C14" s="61"/>
       <c r="D14" s="22" t="s">
         <v>62</v>
       </c>
@@ -10464,8 +10670,8 @@
       <c r="A15" s="22">
         <v>14</v>
       </c>
-      <c r="B15" s="52"/>
-      <c r="C15" s="50"/>
+      <c r="B15" s="62"/>
+      <c r="C15" s="61"/>
       <c r="D15" s="22" t="s">
         <v>64</v>
       </c>
@@ -10489,8 +10695,8 @@
       <c r="A16" s="22">
         <v>15</v>
       </c>
-      <c r="B16" s="52"/>
-      <c r="C16" s="50" t="s">
+      <c r="B16" s="62"/>
+      <c r="C16" s="61" t="s">
         <v>67</v>
       </c>
       <c r="D16" s="22" t="s">
@@ -10516,8 +10722,8 @@
       <c r="A17" s="22">
         <v>16</v>
       </c>
-      <c r="B17" s="52"/>
-      <c r="C17" s="50"/>
+      <c r="B17" s="62"/>
+      <c r="C17" s="61"/>
       <c r="D17" s="22" t="s">
         <v>71</v>
       </c>
@@ -10541,8 +10747,8 @@
       <c r="A18" s="22">
         <v>17</v>
       </c>
-      <c r="B18" s="52"/>
-      <c r="C18" s="50"/>
+      <c r="B18" s="62"/>
+      <c r="C18" s="61"/>
       <c r="D18" s="22" t="s">
         <v>73</v>
       </c>
@@ -10566,8 +10772,8 @@
       <c r="A19" s="22">
         <v>18</v>
       </c>
-      <c r="B19" s="52"/>
-      <c r="C19" s="50" t="s">
+      <c r="B19" s="62"/>
+      <c r="C19" s="61" t="s">
         <v>76</v>
       </c>
       <c r="D19" s="22" t="s">
@@ -10593,8 +10799,8 @@
       <c r="A20" s="22">
         <v>19</v>
       </c>
-      <c r="B20" s="52"/>
-      <c r="C20" s="50"/>
+      <c r="B20" s="62"/>
+      <c r="C20" s="61"/>
       <c r="D20" s="22" t="s">
         <v>80</v>
       </c>
@@ -10618,8 +10824,8 @@
       <c r="A21" s="22">
         <v>20</v>
       </c>
-      <c r="B21" s="52"/>
-      <c r="C21" s="50"/>
+      <c r="B21" s="62"/>
+      <c r="C21" s="61"/>
       <c r="D21" s="22" t="s">
         <v>82</v>
       </c>
@@ -10643,8 +10849,8 @@
       <c r="A22" s="22">
         <v>21</v>
       </c>
-      <c r="B22" s="52"/>
-      <c r="C22" s="50" t="s">
+      <c r="B22" s="62"/>
+      <c r="C22" s="61" t="s">
         <v>85</v>
       </c>
       <c r="D22" s="22" t="s">
@@ -10670,8 +10876,8 @@
       <c r="A23" s="22">
         <v>22</v>
       </c>
-      <c r="B23" s="52"/>
-      <c r="C23" s="50"/>
+      <c r="B23" s="62"/>
+      <c r="C23" s="61"/>
       <c r="D23" s="28" t="s">
         <v>89</v>
       </c>
@@ -10695,8 +10901,8 @@
       <c r="A24" s="22">
         <v>23</v>
       </c>
-      <c r="B24" s="52"/>
-      <c r="C24" s="50"/>
+      <c r="B24" s="62"/>
+      <c r="C24" s="61"/>
       <c r="D24" s="28" t="s">
         <v>91</v>
       </c>
@@ -10720,8 +10926,8 @@
       <c r="A25" s="22">
         <v>24</v>
       </c>
-      <c r="B25" s="52"/>
-      <c r="C25" s="52" t="s">
+      <c r="B25" s="62"/>
+      <c r="C25" s="62" t="s">
         <v>94</v>
       </c>
       <c r="D25" s="28" t="s">
@@ -10747,8 +10953,8 @@
       <c r="A26" s="22">
         <v>25</v>
       </c>
-      <c r="B26" s="52"/>
-      <c r="C26" s="52"/>
+      <c r="B26" s="62"/>
+      <c r="C26" s="62"/>
       <c r="D26" s="28" t="s">
         <v>99</v>
       </c>
@@ -10772,8 +10978,8 @@
       <c r="A27" s="22">
         <v>26</v>
       </c>
-      <c r="B27" s="52"/>
-      <c r="C27" s="52"/>
+      <c r="B27" s="62"/>
+      <c r="C27" s="62"/>
       <c r="D27" s="28" t="s">
         <v>101</v>
       </c>
@@ -10797,8 +11003,8 @@
       <c r="A28" s="22">
         <v>27</v>
       </c>
-      <c r="B28" s="52"/>
-      <c r="C28" s="52" t="s">
+      <c r="B28" s="62"/>
+      <c r="C28" s="62" t="s">
         <v>104</v>
       </c>
       <c r="D28" s="28" t="s">
@@ -10824,8 +11030,8 @@
       <c r="A29" s="22">
         <v>28</v>
       </c>
-      <c r="B29" s="52"/>
-      <c r="C29" s="52"/>
+      <c r="B29" s="62"/>
+      <c r="C29" s="62"/>
       <c r="D29" s="28" t="s">
         <v>108</v>
       </c>
@@ -10849,8 +11055,8 @@
       <c r="A30" s="22">
         <v>29</v>
       </c>
-      <c r="B30" s="52"/>
-      <c r="C30" s="52"/>
+      <c r="B30" s="62"/>
+      <c r="C30" s="62"/>
       <c r="D30" s="28" t="s">
         <v>110</v>
       </c>
@@ -10874,8 +11080,8 @@
       <c r="A31" s="22">
         <v>30</v>
       </c>
-      <c r="B31" s="52"/>
-      <c r="C31" s="52" t="s">
+      <c r="B31" s="62"/>
+      <c r="C31" s="62" t="s">
         <v>113</v>
       </c>
       <c r="D31" s="28" t="s">
@@ -10901,8 +11107,8 @@
       <c r="A32" s="22">
         <v>31</v>
       </c>
-      <c r="B32" s="52"/>
-      <c r="C32" s="52"/>
+      <c r="B32" s="62"/>
+      <c r="C32" s="62"/>
       <c r="D32" s="28" t="s">
         <v>117</v>
       </c>
@@ -10926,8 +11132,8 @@
       <c r="A33" s="22">
         <v>32</v>
       </c>
-      <c r="B33" s="52"/>
-      <c r="C33" s="52"/>
+      <c r="B33" s="62"/>
+      <c r="C33" s="62"/>
       <c r="D33" s="28" t="s">
         <v>119</v>
       </c>
@@ -10951,10 +11157,10 @@
       <c r="A34" s="22">
         <v>33</v>
       </c>
-      <c r="B34" s="50" t="s">
+      <c r="B34" s="61" t="s">
         <v>122</v>
       </c>
-      <c r="C34" s="52" t="s">
+      <c r="C34" s="62" t="s">
         <v>123</v>
       </c>
       <c r="D34" s="28" t="s">
@@ -10980,8 +11186,8 @@
       <c r="A35" s="22">
         <v>34</v>
       </c>
-      <c r="B35" s="50"/>
-      <c r="C35" s="52"/>
+      <c r="B35" s="61"/>
+      <c r="C35" s="62"/>
       <c r="D35" s="22" t="s">
         <v>127</v>
       </c>
@@ -11005,8 +11211,8 @@
       <c r="A36" s="22">
         <v>35</v>
       </c>
-      <c r="B36" s="50"/>
-      <c r="C36" s="52"/>
+      <c r="B36" s="61"/>
+      <c r="C36" s="62"/>
       <c r="D36" s="22" t="s">
         <v>130</v>
       </c>
@@ -11030,8 +11236,8 @@
       <c r="A37" s="22">
         <v>36</v>
       </c>
-      <c r="B37" s="50"/>
-      <c r="C37" s="52" t="s">
+      <c r="B37" s="61"/>
+      <c r="C37" s="62" t="s">
         <v>133</v>
       </c>
       <c r="D37" s="22" t="s">
@@ -11057,8 +11263,8 @@
       <c r="A38" s="22">
         <v>37</v>
       </c>
-      <c r="B38" s="50"/>
-      <c r="C38" s="52"/>
+      <c r="B38" s="61"/>
+      <c r="C38" s="62"/>
       <c r="D38" s="22" t="s">
         <v>137</v>
       </c>
@@ -11082,8 +11288,8 @@
       <c r="A39" s="22">
         <v>38</v>
       </c>
-      <c r="B39" s="50"/>
-      <c r="C39" s="52"/>
+      <c r="B39" s="61"/>
+      <c r="C39" s="62"/>
       <c r="D39" s="22" t="s">
         <v>140</v>
       </c>
@@ -11107,10 +11313,10 @@
       <c r="A40" s="22">
         <v>39</v>
       </c>
-      <c r="B40" s="51" t="s">
+      <c r="B40" s="63" t="s">
         <v>143</v>
       </c>
-      <c r="C40" s="50" t="s">
+      <c r="C40" s="61" t="s">
         <v>144</v>
       </c>
       <c r="D40" s="22" t="s">
@@ -11136,8 +11342,8 @@
       <c r="A41" s="22">
         <v>40</v>
       </c>
-      <c r="B41" s="51"/>
-      <c r="C41" s="50"/>
+      <c r="B41" s="63"/>
+      <c r="C41" s="61"/>
       <c r="D41" s="22" t="s">
         <v>148</v>
       </c>
@@ -11161,8 +11367,8 @@
       <c r="A42" s="22">
         <v>41</v>
       </c>
-      <c r="B42" s="51"/>
-      <c r="C42" s="50" t="s">
+      <c r="B42" s="63"/>
+      <c r="C42" s="61" t="s">
         <v>151</v>
       </c>
       <c r="D42" s="22" t="s">
@@ -11188,8 +11394,8 @@
       <c r="A43" s="22">
         <v>42</v>
       </c>
-      <c r="B43" s="51"/>
-      <c r="C43" s="50"/>
+      <c r="B43" s="63"/>
+      <c r="C43" s="61"/>
       <c r="D43" s="22" t="s">
         <v>155</v>
       </c>
@@ -11213,10 +11419,10 @@
       <c r="A44" s="22">
         <v>43</v>
       </c>
-      <c r="B44" s="51" t="s">
+      <c r="B44" s="63" t="s">
         <v>158</v>
       </c>
-      <c r="C44" s="50" t="s">
+      <c r="C44" s="61" t="s">
         <v>159</v>
       </c>
       <c r="D44" s="22" t="s">
@@ -11242,8 +11448,8 @@
       <c r="A45" s="22">
         <v>44</v>
       </c>
-      <c r="B45" s="51"/>
-      <c r="C45" s="50"/>
+      <c r="B45" s="63"/>
+      <c r="C45" s="61"/>
       <c r="D45" s="22" t="s">
         <v>163</v>
       </c>
@@ -11267,8 +11473,8 @@
       <c r="A46" s="22">
         <v>45</v>
       </c>
-      <c r="B46" s="51"/>
-      <c r="C46" s="50" t="s">
+      <c r="B46" s="63"/>
+      <c r="C46" s="61" t="s">
         <v>166</v>
       </c>
       <c r="D46" s="22" t="s">
@@ -11294,8 +11500,8 @@
       <c r="A47" s="22">
         <v>46</v>
       </c>
-      <c r="B47" s="51"/>
-      <c r="C47" s="50"/>
+      <c r="B47" s="63"/>
+      <c r="C47" s="61"/>
       <c r="D47" s="22" t="s">
         <v>171</v>
       </c>
@@ -11319,10 +11525,10 @@
       <c r="A48" s="31">
         <v>47</v>
       </c>
-      <c r="B48" s="50" t="s">
+      <c r="B48" s="61" t="s">
         <v>174</v>
       </c>
-      <c r="C48" s="50" t="s">
+      <c r="C48" s="61" t="s">
         <v>175</v>
       </c>
       <c r="D48" s="22" t="s">
@@ -11348,8 +11554,8 @@
       <c r="A49" s="22">
         <v>48</v>
       </c>
-      <c r="B49" s="50"/>
-      <c r="C49" s="50"/>
+      <c r="B49" s="61"/>
+      <c r="C49" s="61"/>
       <c r="D49" s="22" t="s">
         <v>179</v>
       </c>
@@ -11373,8 +11579,8 @@
       <c r="A50" s="22">
         <v>49</v>
       </c>
-      <c r="B50" s="50"/>
-      <c r="C50" s="50"/>
+      <c r="B50" s="61"/>
+      <c r="C50" s="61"/>
       <c r="D50" s="22" t="s">
         <v>181</v>
       </c>
@@ -11398,8 +11604,8 @@
       <c r="A51" s="22">
         <v>50</v>
       </c>
-      <c r="B51" s="50"/>
-      <c r="C51" s="50" t="s">
+      <c r="B51" s="61"/>
+      <c r="C51" s="61" t="s">
         <v>184</v>
       </c>
       <c r="D51" s="22" t="s">
@@ -11425,8 +11631,8 @@
       <c r="A52" s="22">
         <v>51</v>
       </c>
-      <c r="B52" s="50"/>
-      <c r="C52" s="50"/>
+      <c r="B52" s="61"/>
+      <c r="C52" s="61"/>
       <c r="D52" s="22" t="s">
         <v>188</v>
       </c>
@@ -11450,8 +11656,8 @@
       <c r="A53" s="22">
         <v>52</v>
       </c>
-      <c r="B53" s="50"/>
-      <c r="C53" s="50"/>
+      <c r="B53" s="61"/>
+      <c r="C53" s="61"/>
       <c r="D53" s="22" t="s">
         <v>190</v>
       </c>
@@ -11475,8 +11681,8 @@
       <c r="A54" s="22">
         <v>53</v>
       </c>
-      <c r="B54" s="50"/>
-      <c r="C54" s="50" t="s">
+      <c r="B54" s="61"/>
+      <c r="C54" s="61" t="s">
         <v>193</v>
       </c>
       <c r="D54" s="22" t="s">
@@ -11502,8 +11708,8 @@
       <c r="A55" s="22">
         <v>54</v>
       </c>
-      <c r="B55" s="50"/>
-      <c r="C55" s="50"/>
+      <c r="B55" s="61"/>
+      <c r="C55" s="61"/>
       <c r="D55" s="22" t="s">
         <v>197</v>
       </c>
@@ -11527,8 +11733,8 @@
       <c r="A56" s="22">
         <v>55</v>
       </c>
-      <c r="B56" s="50"/>
-      <c r="C56" s="50"/>
+      <c r="B56" s="61"/>
+      <c r="C56" s="61"/>
       <c r="D56" s="22" t="s">
         <v>199</v>
       </c>
@@ -11552,8 +11758,8 @@
       <c r="A57" s="22">
         <v>56</v>
       </c>
-      <c r="B57" s="50"/>
-      <c r="C57" s="50" t="s">
+      <c r="B57" s="61"/>
+      <c r="C57" s="61" t="s">
         <v>202</v>
       </c>
       <c r="D57" s="22" t="s">
@@ -11579,8 +11785,8 @@
       <c r="A58" s="22">
         <v>57</v>
       </c>
-      <c r="B58" s="50"/>
-      <c r="C58" s="50"/>
+      <c r="B58" s="61"/>
+      <c r="C58" s="61"/>
       <c r="D58" s="22" t="s">
         <v>206</v>
       </c>
@@ -11604,8 +11810,8 @@
       <c r="A59" s="22">
         <v>58</v>
       </c>
-      <c r="B59" s="50"/>
-      <c r="C59" s="50"/>
+      <c r="B59" s="61"/>
+      <c r="C59" s="61"/>
       <c r="D59" s="22" t="s">
         <v>208</v>
       </c>
@@ -11629,8 +11835,8 @@
       <c r="A60" s="22">
         <v>59</v>
       </c>
-      <c r="B60" s="50"/>
-      <c r="C60" s="50" t="s">
+      <c r="B60" s="61"/>
+      <c r="C60" s="61" t="s">
         <v>211</v>
       </c>
       <c r="D60" s="22" t="s">
@@ -11656,8 +11862,8 @@
       <c r="A61" s="22">
         <v>60</v>
       </c>
-      <c r="B61" s="50"/>
-      <c r="C61" s="50"/>
+      <c r="B61" s="61"/>
+      <c r="C61" s="61"/>
       <c r="D61" s="22" t="s">
         <v>215</v>
       </c>
@@ -11681,8 +11887,8 @@
       <c r="A62" s="22">
         <v>61</v>
       </c>
-      <c r="B62" s="50"/>
-      <c r="C62" s="50"/>
+      <c r="B62" s="61"/>
+      <c r="C62" s="61"/>
       <c r="D62" s="22" t="s">
         <v>217</v>
       </c>
@@ -11706,8 +11912,8 @@
       <c r="A63" s="22">
         <v>62</v>
       </c>
-      <c r="B63" s="50"/>
-      <c r="C63" s="50" t="s">
+      <c r="B63" s="61"/>
+      <c r="C63" s="61" t="s">
         <v>220</v>
       </c>
       <c r="D63" s="22" t="s">
@@ -11733,8 +11939,8 @@
       <c r="A64" s="22">
         <v>63</v>
       </c>
-      <c r="B64" s="50"/>
-      <c r="C64" s="50"/>
+      <c r="B64" s="61"/>
+      <c r="C64" s="61"/>
       <c r="D64" s="28" t="s">
         <v>224</v>
       </c>
@@ -11758,8 +11964,8 @@
       <c r="A65" s="22">
         <v>64</v>
       </c>
-      <c r="B65" s="50"/>
-      <c r="C65" s="50"/>
+      <c r="B65" s="61"/>
+      <c r="C65" s="61"/>
       <c r="D65" s="28" t="s">
         <v>226</v>
       </c>
@@ -11783,8 +11989,8 @@
       <c r="A66" s="22">
         <v>65</v>
       </c>
-      <c r="B66" s="50"/>
-      <c r="C66" s="50" t="s">
+      <c r="B66" s="61"/>
+      <c r="C66" s="61" t="s">
         <v>229</v>
       </c>
       <c r="D66" s="28" t="s">
@@ -11810,8 +12016,8 @@
       <c r="A67" s="22">
         <v>66</v>
       </c>
-      <c r="B67" s="50"/>
-      <c r="C67" s="50"/>
+      <c r="B67" s="61"/>
+      <c r="C67" s="61"/>
       <c r="D67" s="28" t="s">
         <v>233</v>
       </c>
@@ -11835,8 +12041,8 @@
       <c r="A68" s="22">
         <v>67</v>
       </c>
-      <c r="B68" s="50"/>
-      <c r="C68" s="50"/>
+      <c r="B68" s="61"/>
+      <c r="C68" s="61"/>
       <c r="D68" s="28" t="s">
         <v>235</v>
       </c>
@@ -11860,8 +12066,8 @@
       <c r="A69" s="22">
         <v>68</v>
       </c>
-      <c r="B69" s="50"/>
-      <c r="C69" s="50" t="s">
+      <c r="B69" s="61"/>
+      <c r="C69" s="61" t="s">
         <v>238</v>
       </c>
       <c r="D69" s="28" t="s">
@@ -11887,8 +12093,8 @@
       <c r="A70" s="22">
         <v>69</v>
       </c>
-      <c r="B70" s="50"/>
-      <c r="C70" s="50"/>
+      <c r="B70" s="61"/>
+      <c r="C70" s="61"/>
       <c r="D70" s="28" t="s">
         <v>242</v>
       </c>
@@ -11912,8 +12118,8 @@
       <c r="A71" s="22">
         <v>70</v>
       </c>
-      <c r="B71" s="50"/>
-      <c r="C71" s="50"/>
+      <c r="B71" s="61"/>
+      <c r="C71" s="61"/>
       <c r="D71" s="28" t="s">
         <v>244</v>
       </c>
@@ -11937,8 +12143,8 @@
       <c r="A72" s="22">
         <v>71</v>
       </c>
-      <c r="B72" s="50"/>
-      <c r="C72" s="50" t="s">
+      <c r="B72" s="61"/>
+      <c r="C72" s="61" t="s">
         <v>247</v>
       </c>
       <c r="D72" s="28" t="s">
@@ -11964,8 +12170,8 @@
       <c r="A73" s="22">
         <v>72</v>
       </c>
-      <c r="B73" s="50"/>
-      <c r="C73" s="50"/>
+      <c r="B73" s="61"/>
+      <c r="C73" s="61"/>
       <c r="D73" s="28" t="s">
         <v>251</v>
       </c>
@@ -11989,8 +12195,8 @@
       <c r="A74" s="22">
         <v>73</v>
       </c>
-      <c r="B74" s="50"/>
-      <c r="C74" s="50"/>
+      <c r="B74" s="61"/>
+      <c r="C74" s="61"/>
       <c r="D74" s="28" t="s">
         <v>253</v>
       </c>
@@ -12014,10 +12220,10 @@
       <c r="A75" s="22">
         <v>74</v>
       </c>
-      <c r="B75" s="50" t="s">
+      <c r="B75" s="61" t="s">
         <v>256</v>
       </c>
-      <c r="C75" s="50" t="s">
+      <c r="C75" s="61" t="s">
         <v>257</v>
       </c>
       <c r="D75" s="28" t="s">
@@ -12043,8 +12249,8 @@
       <c r="A76" s="22">
         <v>75</v>
       </c>
-      <c r="B76" s="50"/>
-      <c r="C76" s="50"/>
+      <c r="B76" s="61"/>
+      <c r="C76" s="61"/>
       <c r="D76" s="22" t="s">
         <v>261</v>
       </c>
@@ -12068,8 +12274,8 @@
       <c r="A77" s="22">
         <v>76</v>
       </c>
-      <c r="B77" s="50"/>
-      <c r="C77" s="50"/>
+      <c r="B77" s="61"/>
+      <c r="C77" s="61"/>
       <c r="D77" s="22" t="s">
         <v>264</v>
       </c>
@@ -12093,8 +12299,8 @@
       <c r="A78" s="22">
         <v>77</v>
       </c>
-      <c r="B78" s="50"/>
-      <c r="C78" s="51" t="s">
+      <c r="B78" s="61"/>
+      <c r="C78" s="63" t="s">
         <v>267</v>
       </c>
       <c r="D78" s="22" t="s">
@@ -12120,8 +12326,8 @@
       <c r="A79" s="22">
         <v>78</v>
       </c>
-      <c r="B79" s="50"/>
-      <c r="C79" s="51"/>
+      <c r="B79" s="61"/>
+      <c r="C79" s="63"/>
       <c r="D79" s="22" t="s">
         <v>137</v>
       </c>
@@ -12145,8 +12351,8 @@
       <c r="A80" s="22">
         <v>79</v>
       </c>
-      <c r="B80" s="50"/>
-      <c r="C80" s="51"/>
+      <c r="B80" s="61"/>
+      <c r="C80" s="63"/>
       <c r="D80" s="22" t="s">
         <v>140</v>
       </c>
@@ -12170,10 +12376,10 @@
       <c r="A81" s="22">
         <v>80</v>
       </c>
-      <c r="B81" s="50" t="s">
+      <c r="B81" s="61" t="s">
         <v>274</v>
       </c>
-      <c r="C81" s="50" t="s">
+      <c r="C81" s="61" t="s">
         <v>275</v>
       </c>
       <c r="D81" s="22" t="s">
@@ -12199,8 +12405,8 @@
       <c r="A82" s="22">
         <v>81</v>
       </c>
-      <c r="B82" s="50"/>
-      <c r="C82" s="50"/>
+      <c r="B82" s="61"/>
+      <c r="C82" s="61"/>
       <c r="D82" s="22" t="s">
         <v>279</v>
       </c>
@@ -12224,8 +12430,8 @@
       <c r="A83" s="22">
         <v>82</v>
       </c>
-      <c r="B83" s="50"/>
-      <c r="C83" s="51" t="s">
+      <c r="B83" s="61"/>
+      <c r="C83" s="63" t="s">
         <v>282</v>
       </c>
       <c r="D83" s="22" t="s">
@@ -12251,8 +12457,8 @@
       <c r="A84" s="22">
         <v>83</v>
       </c>
-      <c r="B84" s="50"/>
-      <c r="C84" s="51"/>
+      <c r="B84" s="61"/>
+      <c r="C84" s="63"/>
       <c r="D84" s="22" t="s">
         <v>286</v>
       </c>
@@ -12276,10 +12482,10 @@
       <c r="A85" s="22">
         <v>84</v>
       </c>
-      <c r="B85" s="50" t="s">
+      <c r="B85" s="61" t="s">
         <v>289</v>
       </c>
-      <c r="C85" s="50" t="s">
+      <c r="C85" s="61" t="s">
         <v>290</v>
       </c>
       <c r="D85" s="22" t="s">
@@ -12305,8 +12511,8 @@
       <c r="A86" s="22">
         <v>85</v>
       </c>
-      <c r="B86" s="50"/>
-      <c r="C86" s="50"/>
+      <c r="B86" s="61"/>
+      <c r="C86" s="61"/>
       <c r="D86" s="22" t="s">
         <v>294</v>
       </c>
@@ -12330,8 +12536,8 @@
       <c r="A87" s="22">
         <v>86</v>
       </c>
-      <c r="B87" s="50"/>
-      <c r="C87" s="50" t="s">
+      <c r="B87" s="61"/>
+      <c r="C87" s="61" t="s">
         <v>297</v>
       </c>
       <c r="D87" s="22" t="s">
@@ -12357,8 +12563,8 @@
       <c r="A88" s="22">
         <v>87</v>
       </c>
-      <c r="B88" s="50"/>
-      <c r="C88" s="50"/>
+      <c r="B88" s="61"/>
+      <c r="C88" s="61"/>
       <c r="D88" s="22" t="s">
         <v>301</v>
       </c>
@@ -12382,10 +12588,10 @@
       <c r="A89" s="22">
         <v>88</v>
       </c>
-      <c r="B89" s="50" t="s">
+      <c r="B89" s="61" t="s">
         <v>304</v>
       </c>
-      <c r="C89" s="50" t="s">
+      <c r="C89" s="61" t="s">
         <v>305</v>
       </c>
       <c r="D89" s="22" t="s">
@@ -12411,8 +12617,8 @@
       <c r="A90" s="22">
         <v>89</v>
       </c>
-      <c r="B90" s="50"/>
-      <c r="C90" s="50"/>
+      <c r="B90" s="61"/>
+      <c r="C90" s="61"/>
       <c r="D90" s="22" t="s">
         <v>310</v>
       </c>
@@ -12436,8 +12642,8 @@
       <c r="A91" s="22">
         <v>90</v>
       </c>
-      <c r="B91" s="50"/>
-      <c r="C91" s="50"/>
+      <c r="B91" s="61"/>
+      <c r="C91" s="61"/>
       <c r="D91" s="25" t="s">
         <v>313</v>
       </c>
@@ -12461,8 +12667,8 @@
       <c r="A92" s="22">
         <v>91</v>
       </c>
-      <c r="B92" s="50"/>
-      <c r="C92" s="50" t="s">
+      <c r="B92" s="61"/>
+      <c r="C92" s="61" t="s">
         <v>316</v>
       </c>
       <c r="D92" s="25" t="s">
@@ -12488,8 +12694,8 @@
       <c r="A93" s="22">
         <v>92</v>
       </c>
-      <c r="B93" s="50"/>
-      <c r="C93" s="50"/>
+      <c r="B93" s="61"/>
+      <c r="C93" s="61"/>
       <c r="D93" s="25" t="s">
         <v>320</v>
       </c>
@@ -12511,8 +12717,8 @@
     </row>
     <row r="94" spans="1:9" ht="113.25" customHeight="1">
       <c r="A94" s="22"/>
-      <c r="B94" s="50"/>
-      <c r="C94" s="50"/>
+      <c r="B94" s="61"/>
+      <c r="C94" s="61"/>
       <c r="D94" s="25"/>
       <c r="E94" s="37"/>
       <c r="F94" s="22"/>
@@ -12524,8 +12730,8 @@
       <c r="A95" s="22">
         <v>93</v>
       </c>
-      <c r="B95" s="50"/>
-      <c r="C95" s="50"/>
+      <c r="B95" s="61"/>
+      <c r="C95" s="61"/>
       <c r="D95" s="25" t="s">
         <v>323</v>
       </c>
@@ -12549,7 +12755,7 @@
       <c r="A96" s="22">
         <v>94</v>
       </c>
-      <c r="B96" s="50" t="s">
+      <c r="B96" s="61" t="s">
         <v>326</v>
       </c>
       <c r="C96" s="22" t="s">
@@ -12578,7 +12784,7 @@
       <c r="A97" s="22">
         <v>95</v>
       </c>
-      <c r="B97" s="50"/>
+      <c r="B97" s="61"/>
       <c r="C97" s="22" t="s">
         <v>332</v>
       </c>
@@ -12605,7 +12811,7 @@
       <c r="A98" s="22">
         <v>96</v>
       </c>
-      <c r="B98" s="50"/>
+      <c r="B98" s="61"/>
       <c r="C98" s="22" t="s">
         <v>336</v>
       </c>
@@ -12632,10 +12838,10 @@
       <c r="A99" s="8">
         <v>97</v>
       </c>
-      <c r="B99" s="54" t="s">
+      <c r="B99" s="58" t="s">
         <v>256</v>
       </c>
-      <c r="C99" s="53" t="s">
+      <c r="C99" s="57" t="s">
         <v>340</v>
       </c>
       <c r="D99" s="6" t="s">
@@ -12661,8 +12867,8 @@
       <c r="A100" s="8">
         <v>98</v>
       </c>
-      <c r="B100" s="54"/>
-      <c r="C100" s="53"/>
+      <c r="B100" s="58"/>
+      <c r="C100" s="57"/>
       <c r="D100" s="6" t="s">
         <v>344</v>
       </c>
@@ -12686,8 +12892,8 @@
       <c r="A101" s="8">
         <v>99</v>
       </c>
-      <c r="B101" s="54"/>
-      <c r="C101" s="53"/>
+      <c r="B101" s="58"/>
+      <c r="C101" s="57"/>
       <c r="D101" s="8" t="s">
         <v>347</v>
       </c>
@@ -12711,8 +12917,8 @@
       <c r="A102" s="8">
         <v>100</v>
       </c>
-      <c r="B102" s="54"/>
-      <c r="C102" s="53"/>
+      <c r="B102" s="58"/>
+      <c r="C102" s="57"/>
       <c r="D102" s="8" t="s">
         <v>350</v>
       </c>
@@ -12736,8 +12942,8 @@
       <c r="A103" s="8">
         <v>101</v>
       </c>
-      <c r="B103" s="54"/>
-      <c r="C103" s="53"/>
+      <c r="B103" s="58"/>
+      <c r="C103" s="57"/>
       <c r="D103" s="8" t="s">
         <v>353</v>
       </c>
@@ -12761,8 +12967,8 @@
       <c r="A104" s="8">
         <v>102</v>
       </c>
-      <c r="B104" s="54"/>
-      <c r="C104" s="53"/>
+      <c r="B104" s="58"/>
+      <c r="C104" s="57"/>
       <c r="D104" s="8" t="s">
         <v>356</v>
       </c>
@@ -12780,8 +12986,8 @@
       <c r="A105" s="8">
         <v>103</v>
       </c>
-      <c r="B105" s="54"/>
-      <c r="C105" s="53"/>
+      <c r="B105" s="58"/>
+      <c r="C105" s="57"/>
       <c r="D105" s="8" t="s">
         <v>350</v>
       </c>
@@ -12805,10 +13011,10 @@
       <c r="A106" s="8">
         <v>104</v>
       </c>
-      <c r="B106" s="56" t="s">
+      <c r="B106" s="60" t="s">
         <v>274</v>
       </c>
-      <c r="C106" s="55" t="s">
+      <c r="C106" s="59" t="s">
         <v>360</v>
       </c>
       <c r="D106" s="8" t="s">
@@ -12834,8 +13040,8 @@
       <c r="A107" s="8">
         <v>105</v>
       </c>
-      <c r="B107" s="56"/>
-      <c r="C107" s="55"/>
+      <c r="B107" s="60"/>
+      <c r="C107" s="59"/>
       <c r="D107" s="8" t="s">
         <v>364</v>
       </c>
@@ -12859,8 +13065,8 @@
       <c r="A108" s="8">
         <v>106</v>
       </c>
-      <c r="B108" s="56"/>
-      <c r="C108" s="55"/>
+      <c r="B108" s="60"/>
+      <c r="C108" s="59"/>
       <c r="D108" s="8" t="s">
         <v>367</v>
       </c>
@@ -12884,8 +13090,8 @@
       <c r="A109" s="8">
         <v>107</v>
       </c>
-      <c r="B109" s="56"/>
-      <c r="C109" s="55"/>
+      <c r="B109" s="60"/>
+      <c r="C109" s="59"/>
       <c r="D109" s="8" t="s">
         <v>370</v>
       </c>
@@ -12909,10 +13115,10 @@
       <c r="A110" s="8">
         <v>108</v>
       </c>
-      <c r="B110" s="56" t="s">
+      <c r="B110" s="60" t="s">
         <v>289</v>
       </c>
-      <c r="C110" s="55" t="s">
+      <c r="C110" s="59" t="s">
         <v>373</v>
       </c>
       <c r="D110" s="8" t="s">
@@ -12938,8 +13144,8 @@
       <c r="A111" s="8">
         <v>109</v>
       </c>
-      <c r="B111" s="56"/>
-      <c r="C111" s="55"/>
+      <c r="B111" s="60"/>
+      <c r="C111" s="59"/>
       <c r="D111" s="8" t="s">
         <v>377</v>
       </c>
@@ -12963,8 +13169,8 @@
       <c r="A112" s="8">
         <v>110</v>
       </c>
-      <c r="B112" s="56"/>
-      <c r="C112" s="55"/>
+      <c r="B112" s="60"/>
+      <c r="C112" s="59"/>
       <c r="D112" s="8" t="s">
         <v>380</v>
       </c>
@@ -12988,8 +13194,8 @@
       <c r="A113" s="8">
         <v>111</v>
       </c>
-      <c r="B113" s="56"/>
-      <c r="C113" s="55"/>
+      <c r="B113" s="60"/>
+      <c r="C113" s="59"/>
       <c r="D113" s="8" t="s">
         <v>383</v>
       </c>
@@ -13011,12 +13217,34 @@
     </row>
   </sheetData>
   <mergeCells count="50">
-    <mergeCell ref="C99:C105"/>
-    <mergeCell ref="B99:B105"/>
-    <mergeCell ref="C106:C109"/>
-    <mergeCell ref="B106:B109"/>
-    <mergeCell ref="C110:C113"/>
-    <mergeCell ref="B110:B113"/>
+    <mergeCell ref="B96:B98"/>
+    <mergeCell ref="B75:B80"/>
+    <mergeCell ref="B81:B84"/>
+    <mergeCell ref="B85:B88"/>
+    <mergeCell ref="B89:B95"/>
+    <mergeCell ref="C87:C88"/>
+    <mergeCell ref="C89:C91"/>
+    <mergeCell ref="C92:C95"/>
+    <mergeCell ref="C63:C65"/>
+    <mergeCell ref="C66:C68"/>
+    <mergeCell ref="C69:C71"/>
+    <mergeCell ref="C72:C74"/>
+    <mergeCell ref="C75:C77"/>
+    <mergeCell ref="C78:C80"/>
+    <mergeCell ref="C81:C82"/>
+    <mergeCell ref="C83:C84"/>
+    <mergeCell ref="C85:C86"/>
+    <mergeCell ref="C48:C50"/>
+    <mergeCell ref="C51:C53"/>
+    <mergeCell ref="C54:C56"/>
+    <mergeCell ref="C57:C59"/>
+    <mergeCell ref="C60:C62"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="B4:B6"/>
+    <mergeCell ref="C7:C9"/>
+    <mergeCell ref="C10:C12"/>
+    <mergeCell ref="C13:C15"/>
+    <mergeCell ref="B7:B33"/>
     <mergeCell ref="B48:B74"/>
     <mergeCell ref="C16:C18"/>
     <mergeCell ref="C19:C21"/>
@@ -13033,34 +13261,12 @@
     <mergeCell ref="B40:B43"/>
     <mergeCell ref="C40:C41"/>
     <mergeCell ref="C42:C43"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="B4:B6"/>
-    <mergeCell ref="C7:C9"/>
-    <mergeCell ref="C10:C12"/>
-    <mergeCell ref="C13:C15"/>
-    <mergeCell ref="B7:B33"/>
-    <mergeCell ref="C48:C50"/>
-    <mergeCell ref="C51:C53"/>
-    <mergeCell ref="C54:C56"/>
-    <mergeCell ref="C57:C59"/>
-    <mergeCell ref="C60:C62"/>
-    <mergeCell ref="C87:C88"/>
-    <mergeCell ref="C89:C91"/>
-    <mergeCell ref="C92:C95"/>
-    <mergeCell ref="C63:C65"/>
-    <mergeCell ref="C66:C68"/>
-    <mergeCell ref="C69:C71"/>
-    <mergeCell ref="C72:C74"/>
-    <mergeCell ref="C75:C77"/>
-    <mergeCell ref="C78:C80"/>
-    <mergeCell ref="C81:C82"/>
-    <mergeCell ref="C83:C84"/>
-    <mergeCell ref="C85:C86"/>
-    <mergeCell ref="B96:B98"/>
-    <mergeCell ref="B75:B80"/>
-    <mergeCell ref="B81:B84"/>
-    <mergeCell ref="B85:B88"/>
-    <mergeCell ref="B89:B95"/>
+    <mergeCell ref="C99:C105"/>
+    <mergeCell ref="B99:B105"/>
+    <mergeCell ref="C106:C109"/>
+    <mergeCell ref="B106:B109"/>
+    <mergeCell ref="C110:C113"/>
+    <mergeCell ref="B110:B113"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13068,16 +13274,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE6FFABF-1821-4175-95EA-105A738029C5}">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="2" max="2" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38" customWidth="1"/>
     <col min="3" max="3" width="51.5703125" customWidth="1"/>
-    <col min="4" max="4" width="36.5703125" customWidth="1"/>
+    <col min="4" max="4" width="58.7109375" customWidth="1"/>
     <col min="5" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:6">
       <c r="A1" s="49" t="s">
         <v>386</v>
       </c>
@@ -13090,212 +13296,385 @@
       <c r="D1" s="49" t="s">
         <v>389</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="115.5">
+      <c r="E1" s="64" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="64" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="86.25" customHeight="1">
       <c r="A2" s="8">
         <v>1</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C2" s="40" t="s">
-        <v>391</v>
-      </c>
-      <c r="D2" s="40" t="s">
         <v>392</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="130.5">
+      <c r="D2" s="65" t="s">
+        <v>393</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>394</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="110.25" customHeight="1">
       <c r="A3" s="8">
         <v>2</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="C3" s="40" t="s">
+        <v>396</v>
+      </c>
+      <c r="D3" s="65" t="s">
+        <v>397</v>
+      </c>
+      <c r="E3" s="8" t="s">
         <v>394</v>
       </c>
-      <c r="D3" s="40" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="130.5">
+      <c r="F3" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="114.75" customHeight="1">
       <c r="A4" s="8">
         <v>3</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="C4" s="40" t="s">
-        <v>397</v>
-      </c>
-      <c r="D4" s="40" t="s">
-        <v>398</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="130.5">
+        <v>399</v>
+      </c>
+      <c r="D4" s="65" t="s">
+        <v>400</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>394</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="120" customHeight="1">
       <c r="A5" s="8">
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="C5" s="40" t="s">
-        <v>400</v>
-      </c>
-      <c r="D5" s="40" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="130.5">
+        <v>402</v>
+      </c>
+      <c r="D5" s="65" t="s">
+        <v>403</v>
+      </c>
+      <c r="E5" s="68">
+        <v>46028</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="130.5">
       <c r="A6" s="8">
         <v>5</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="C6" s="40" t="s">
-        <v>403</v>
-      </c>
-      <c r="D6" s="40" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="130.5">
+        <v>405</v>
+      </c>
+      <c r="D6" s="65" t="s">
+        <v>406</v>
+      </c>
+      <c r="E6" s="68">
+        <v>46028</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="130.5">
       <c r="A7" s="8">
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="C7" s="40" t="s">
-        <v>406</v>
-      </c>
-      <c r="D7" s="40" t="s">
-        <v>407</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="130.5">
+        <v>408</v>
+      </c>
+      <c r="D7" s="65" t="s">
+        <v>409</v>
+      </c>
+      <c r="E7" s="68">
+        <v>46028</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="130.5">
       <c r="A8" s="8">
         <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
       <c r="C8" s="40" t="s">
-        <v>409</v>
-      </c>
-      <c r="D8" s="40" t="s">
         <v>410</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="130.5">
+      <c r="D8" s="65" t="s">
+        <v>411</v>
+      </c>
+      <c r="E8" s="68">
+        <v>46059</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="77.25" customHeight="1">
       <c r="A9" s="8">
         <v>8</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>408</v>
-      </c>
-      <c r="C9" s="40" t="s">
-        <v>411</v>
-      </c>
-      <c r="D9" s="40" t="s">
         <v>412</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="130.5">
+      <c r="C9" s="22" t="s">
+        <v>413</v>
+      </c>
+      <c r="D9" s="65" t="s">
+        <v>414</v>
+      </c>
+      <c r="E9" s="68">
+        <v>46059</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="243.75" customHeight="1">
       <c r="A10" s="8">
+        <v>9</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>415</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>416</v>
+      </c>
+      <c r="D10" s="66" t="s">
+        <v>417</v>
+      </c>
+      <c r="E10" s="68">
+        <v>46059</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="102.75" customHeight="1">
+      <c r="A11" s="8">
+        <v>10</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>418</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>419</v>
+      </c>
+      <c r="D11" s="65" t="s">
+        <v>420</v>
+      </c>
+      <c r="E11" s="68">
+        <v>46087</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="133.5" customHeight="1">
+      <c r="A12" s="8">
+        <v>11</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>421</v>
+      </c>
+      <c r="C12" s="50" t="s">
+        <v>422</v>
+      </c>
+      <c r="D12" s="66" t="s">
+        <v>423</v>
+      </c>
+      <c r="E12" s="68">
+        <v>46087</v>
+      </c>
+      <c r="F12" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="112.5" customHeight="1">
+      <c r="A13" s="8">
         <v>12</v>
       </c>
-      <c r="B10" s="8" t="s">
-        <v>413</v>
-      </c>
-      <c r="C10" s="40" t="s">
-        <v>414</v>
-      </c>
-      <c r="D10" s="40" t="s">
-        <v>415</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="109.5" customHeight="1">
-      <c r="A11" s="8">
+      <c r="B13" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="C13" s="22" t="s">
+        <v>425</v>
+      </c>
+      <c r="D13" s="66" t="s">
+        <v>426</v>
+      </c>
+      <c r="E13" s="68">
+        <v>46087</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="132.75" customHeight="1">
+      <c r="A14" s="52">
         <v>13</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>416</v>
-      </c>
-      <c r="C11" s="40" t="s">
-        <v>417</v>
-      </c>
-      <c r="D11" s="40" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4"/>
-    <row r="18" spans="1:3" ht="141.75" customHeight="1">
-      <c r="A18" s="8"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="37"/>
-    </row>
-    <row r="19" spans="1:3" ht="150" customHeight="1">
-      <c r="A19" s="8"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="40"/>
-    </row>
-    <row r="20" spans="1:3" ht="134.25" customHeight="1">
-      <c r="A20" s="8"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="40"/>
-    </row>
-    <row r="21" spans="1:3" ht="136.5" customHeight="1">
-      <c r="A21" s="8"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="40"/>
-    </row>
-    <row r="22" spans="1:3" ht="159.75" customHeight="1">
-      <c r="A22" s="8"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="40"/>
-    </row>
-    <row r="23" spans="1:3" ht="153.75" customHeight="1">
-      <c r="A23" s="8"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="40"/>
-    </row>
-    <row r="24" spans="1:3" ht="129" customHeight="1">
-      <c r="A24" s="8"/>
-      <c r="B24" s="8"/>
-      <c r="C24" s="40"/>
-    </row>
-    <row r="25" spans="1:3" ht="134.25" customHeight="1">
-      <c r="A25" s="8"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="40"/>
-    </row>
-    <row r="26" spans="1:3" ht="126.75" customHeight="1">
-      <c r="A26" s="8"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="40"/>
-    </row>
-    <row r="27" spans="1:3" ht="149.25" customHeight="1">
-      <c r="A27" s="8"/>
-      <c r="B27" s="8"/>
-      <c r="C27" s="40"/>
-    </row>
-    <row r="28" spans="1:3" ht="144.75" customHeight="1">
-      <c r="A28" s="8"/>
-      <c r="B28" s="8"/>
-      <c r="C28" s="40"/>
-    </row>
-    <row r="29" spans="1:3" ht="146.25" customHeight="1">
-      <c r="A29" s="8"/>
-      <c r="B29" s="8"/>
-      <c r="C29" s="40"/>
-    </row>
-    <row r="30" spans="1:3" ht="123.75" customHeight="1">
-      <c r="A30" s="8"/>
-      <c r="B30" s="8"/>
-      <c r="C30" s="40"/>
+      <c r="B14" s="52" t="s">
+        <v>427</v>
+      </c>
+      <c r="C14" s="55" t="s">
+        <v>428</v>
+      </c>
+      <c r="D14" s="67" t="s">
+        <v>429</v>
+      </c>
+      <c r="E14" s="68">
+        <v>46087</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="83.25" customHeight="1">
+      <c r="A15" s="52">
+        <v>14</v>
+      </c>
+      <c r="B15" s="52" t="s">
+        <v>430</v>
+      </c>
+      <c r="C15" s="56" t="s">
+        <v>431</v>
+      </c>
+      <c r="D15" s="67" t="s">
+        <v>432</v>
+      </c>
+      <c r="E15" s="68">
+        <v>46118</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="107.25" customHeight="1">
+      <c r="A16" s="8">
+        <v>15</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>433</v>
+      </c>
+      <c r="C16" s="25" t="s">
+        <v>434</v>
+      </c>
+      <c r="D16" s="65" t="s">
+        <v>435</v>
+      </c>
+      <c r="E16" s="69" t="s">
+        <v>436</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="107.25" customHeight="1">
+      <c r="A17" s="8">
+        <v>16</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>437</v>
+      </c>
+      <c r="C17" s="25" t="s">
+        <v>438</v>
+      </c>
+      <c r="D17" s="65" t="s">
+        <v>439</v>
+      </c>
+      <c r="E17" s="68">
+        <v>46118</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="141.75" customHeight="1">
+      <c r="A18" s="51"/>
+      <c r="C18" s="54"/>
+      <c r="D18" s="50"/>
+    </row>
+    <row r="19" spans="1:6" ht="150" customHeight="1">
+      <c r="A19" s="51"/>
+      <c r="C19" s="53"/>
+    </row>
+    <row r="20" spans="1:6" ht="134.25" customHeight="1">
+      <c r="A20" s="11"/>
+      <c r="C20" s="53"/>
+    </row>
+    <row r="21" spans="1:6" ht="136.5" customHeight="1">
+      <c r="A21" s="11"/>
+      <c r="C21" s="53"/>
+    </row>
+    <row r="22" spans="1:6" ht="159.75" customHeight="1">
+      <c r="A22" s="11"/>
+      <c r="C22" s="53"/>
+    </row>
+    <row r="23" spans="1:6" ht="153.75" customHeight="1">
+      <c r="A23" s="11"/>
+      <c r="C23" s="53"/>
+    </row>
+    <row r="24" spans="1:6" ht="129" customHeight="1">
+      <c r="A24" s="11"/>
+      <c r="C24" s="53"/>
+    </row>
+    <row r="25" spans="1:6" ht="134.25" customHeight="1">
+      <c r="A25" s="11"/>
+      <c r="C25" s="53"/>
+    </row>
+    <row r="26" spans="1:6" ht="126.75" customHeight="1">
+      <c r="A26" s="11"/>
+      <c r="C26" s="53"/>
+    </row>
+    <row r="27" spans="1:6" ht="149.25" customHeight="1">
+      <c r="A27" s="11"/>
+      <c r="C27" s="53"/>
+    </row>
+    <row r="28" spans="1:6" ht="144.75" customHeight="1">
+      <c r="A28" s="11"/>
+      <c r="C28" s="53"/>
+    </row>
+    <row r="29" spans="1:6" ht="146.25" customHeight="1">
+      <c r="A29" s="11"/>
+      <c r="C29" s="53"/>
+    </row>
+    <row r="30" spans="1:6" ht="123.75" customHeight="1">
+      <c r="A30" s="11"/>
+      <c r="C30" s="53"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -13317,66 +13696,66 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="5" t="s">
-        <v>419</v>
+        <v>440</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>420</v>
+        <v>441</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>419</v>
+        <v>440</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>420</v>
+        <v>441</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>14</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>420</v>
+        <v>441</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="56" t="s">
-        <v>421</v>
-      </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
+      <c r="B2" s="60" t="s">
+        <v>442</v>
+      </c>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
       <c r="F2" s="11"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="54" t="s">
-        <v>422</v>
-      </c>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
+      <c r="B3" s="58" t="s">
+        <v>443</v>
+      </c>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
       <c r="F3" s="11"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="6" t="s">
-        <v>423</v>
+        <v>444</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>425</v>
+        <v>446</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>426</v>
+        <v>447</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -13384,19 +13763,19 @@
         <v>39</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>428</v>
+        <v>449</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>429</v>
+        <v>450</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -13404,19 +13783,19 @@
         <v>50</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>430</v>
+        <v>451</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>431</v>
+        <v>452</v>
       </c>
       <c r="F6" s="11" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -13424,19 +13803,19 @@
         <v>59</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>432</v>
+        <v>453</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>433</v>
+        <v>454</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -13444,19 +13823,19 @@
         <v>68</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>434</v>
+        <v>455</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>435</v>
+        <v>456</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -13464,513 +13843,513 @@
         <v>77</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>436</v>
+        <v>457</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>437</v>
+        <v>458</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="9" t="s">
-        <v>438</v>
+        <v>459</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>439</v>
+        <v>460</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>440</v>
+        <v>461</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>441</v>
+        <v>462</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="9" t="s">
-        <v>442</v>
+        <v>463</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>439</v>
+        <v>460</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>443</v>
+        <v>464</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>444</v>
+        <v>465</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="9" t="s">
+        <v>466</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>448</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>467</v>
+      </c>
+      <c r="D12" s="9" t="s">
         <v>445</v>
       </c>
-      <c r="B12" s="9" t="s">
-        <v>427</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>446</v>
-      </c>
-      <c r="D12" s="9" t="s">
-        <v>424</v>
-      </c>
       <c r="E12" s="8" t="s">
-        <v>447</v>
+        <v>468</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="9" t="s">
+        <v>469</v>
+      </c>
+      <c r="B13" s="9" t="s">
         <v>448</v>
       </c>
-      <c r="B13" s="9" t="s">
-        <v>427</v>
-      </c>
       <c r="C13" s="8" t="s">
-        <v>449</v>
+        <v>470</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>450</v>
+        <v>471</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>451</v>
+        <v>472</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="14.45" customHeight="1">
       <c r="A14" s="20" t="s">
-        <v>452</v>
+        <v>473</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>453</v>
+        <v>474</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>454</v>
+        <v>475</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>451</v>
+        <v>472</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="14.45" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>455</v>
+        <v>476</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>456</v>
+        <v>477</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>457</v>
+        <v>478</v>
       </c>
       <c r="F15" s="11" t="s">
-        <v>451</v>
+        <v>472</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="14.45" customHeight="1">
       <c r="A16" s="16"/>
       <c r="B16" s="18"/>
       <c r="C16" s="8" t="s">
-        <v>458</v>
+        <v>479</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>459</v>
+        <v>480</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>451</v>
+        <v>472</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="14.45" customHeight="1">
       <c r="A17" s="16"/>
       <c r="B17" s="18"/>
       <c r="C17" s="8" t="s">
-        <v>460</v>
+        <v>481</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>461</v>
+        <v>482</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>451</v>
+        <v>472</v>
       </c>
     </row>
     <row r="18" spans="1:6" ht="14.45" customHeight="1">
       <c r="A18" s="16"/>
       <c r="B18" s="18"/>
       <c r="C18" s="9" t="s">
-        <v>462</v>
+        <v>483</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>463</v>
+        <v>484</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>451</v>
+        <v>472</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="14.45" customHeight="1">
       <c r="A19" s="17"/>
       <c r="B19" s="19"/>
       <c r="C19" s="9" t="s">
-        <v>464</v>
+        <v>485</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>424</v>
+        <v>445</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>465</v>
+        <v>486</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>451</v>
+        <v>472</v>
       </c>
     </row>
     <row r="20" spans="1:6" s="15" customFormat="1">
       <c r="A20" s="12" t="s">
-        <v>466</v>
+        <v>487</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>419</v>
+        <v>440</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>467</v>
+        <v>488</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>419</v>
+        <v>440</v>
       </c>
       <c r="E20" s="14" t="s">
-        <v>467</v>
+        <v>488</v>
       </c>
       <c r="F20" s="14" t="s">
-        <v>419</v>
+        <v>440</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="6" t="s">
-        <v>468</v>
+        <v>489</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C21" t="s">
-        <v>469</v>
+        <v>490</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E21" t="s">
-        <v>470</v>
+        <v>491</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="7" t="s">
-        <v>471</v>
+        <v>492</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C22" t="s">
-        <v>472</v>
+        <v>493</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E22" t="s">
-        <v>473</v>
+        <v>494</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="7" t="s">
-        <v>474</v>
+        <v>495</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C23" t="s">
-        <v>475</v>
+        <v>496</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E23" t="s">
-        <v>476</v>
+        <v>497</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="6" t="s">
-        <v>477</v>
+        <v>498</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C24" t="s">
-        <v>478</v>
+        <v>499</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E24" t="s">
-        <v>479</v>
+        <v>500</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="6" t="s">
-        <v>480</v>
+        <v>501</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C25" t="s">
-        <v>481</v>
+        <v>502</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E25" t="s">
-        <v>482</v>
+        <v>503</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="9" t="s">
-        <v>483</v>
+        <v>504</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C26" t="s">
-        <v>484</v>
+        <v>505</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E26" t="s">
-        <v>485</v>
+        <v>506</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="9" t="s">
-        <v>486</v>
+        <v>507</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C27" t="s">
-        <v>487</v>
+        <v>508</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E27" t="s">
-        <v>488</v>
+        <v>509</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="9" t="s">
-        <v>489</v>
+        <v>510</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C28" t="s">
-        <v>490</v>
+        <v>511</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E28" t="s">
-        <v>491</v>
+        <v>512</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="9" t="s">
-        <v>492</v>
+        <v>513</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C29" t="s">
-        <v>493</v>
+        <v>514</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E29" t="s">
-        <v>494</v>
+        <v>515</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="30" spans="1:6">
       <c r="A30" s="1" t="s">
-        <v>495</v>
+        <v>516</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>496</v>
+        <v>517</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>497</v>
+        <v>518</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="1" t="s">
-        <v>498</v>
+        <v>519</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>499</v>
+        <v>520</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>500</v>
+        <v>521</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="1" t="s">
-        <v>501</v>
+        <v>522</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>502</v>
+        <v>523</v>
       </c>
       <c r="C32" t="s">
-        <v>503</v>
+        <v>524</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>504</v>
+        <v>525</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="1" t="s">
-        <v>505</v>
+        <v>526</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>502</v>
+        <v>523</v>
       </c>
       <c r="C33" t="s">
-        <v>506</v>
+        <v>527</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>507</v>
+        <v>528</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="9"/>
       <c r="C34" s="1" t="s">
-        <v>508</v>
+        <v>529</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>509</v>
+        <v>530</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="9"/>
       <c r="C35" s="1" t="s">
-        <v>510</v>
+        <v>531</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>511</v>
+        <v>532</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -13978,13 +14357,13 @@
         <v>323</v>
       </c>
       <c r="D36" t="s">
-        <v>502</v>
+        <v>523</v>
       </c>
       <c r="E36" t="s">
-        <v>512</v>
+        <v>533</v>
       </c>
       <c r="F36" t="s">
-        <v>502</v>
+        <v>523</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -13992,30 +14371,30 @@
         <v>313</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>502</v>
+        <v>523</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>513</v>
+        <v>534</v>
       </c>
       <c r="F37" t="s">
-        <v>502</v>
+        <v>523</v>
       </c>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="33" t="s">
-        <v>514</v>
+        <v>535</v>
       </c>
       <c r="B38" s="34" t="s">
         <v>14</v>
       </c>
       <c r="C38" s="35" t="s">
-        <v>515</v>
+        <v>536</v>
       </c>
       <c r="D38" s="35" t="s">
         <v>14</v>
       </c>
       <c r="E38" s="36" t="s">
-        <v>514</v>
+        <v>535</v>
       </c>
       <c r="F38" s="36" t="s">
         <v>14</v>
@@ -14026,19 +14405,19 @@
         <v>341</v>
       </c>
       <c r="B39" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>344</v>
       </c>
       <c r="D39" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>347</v>
       </c>
       <c r="F39" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="15" customHeight="1">
@@ -14046,19 +14425,19 @@
         <v>350</v>
       </c>
       <c r="B40" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="C40" t="s">
         <v>353</v>
       </c>
       <c r="D40" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E40" t="s">
         <v>356</v>
       </c>
       <c r="F40" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="15" customHeight="1">
@@ -14066,13 +14445,13 @@
         <v>361</v>
       </c>
       <c r="D41" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E41" t="s">
         <v>364</v>
       </c>
       <c r="F41" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="15" customHeight="1">
@@ -14080,13 +14459,13 @@
         <v>367</v>
       </c>
       <c r="D42" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E42" t="s">
         <v>370</v>
       </c>
       <c r="F42" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="15" customHeight="1">
@@ -14094,13 +14473,13 @@
         <v>374</v>
       </c>
       <c r="D43" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E43" t="s">
         <v>377</v>
       </c>
       <c r="F43" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="15" customHeight="1">
@@ -14108,13 +14487,13 @@
         <v>380</v>
       </c>
       <c r="D44" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
       <c r="E44" t="s">
         <v>383</v>
       </c>
       <c r="F44" t="s">
-        <v>427</v>
+        <v>448</v>
       </c>
     </row>
   </sheetData>
@@ -14140,19 +14519,19 @@
   <sheetData>
     <row r="1" spans="1:24">
       <c r="A1" s="38" t="s">
-        <v>516</v>
+        <v>537</v>
       </c>
       <c r="B1" s="38" t="s">
-        <v>517</v>
+        <v>538</v>
       </c>
       <c r="C1" s="39" t="s">
-        <v>518</v>
+        <v>539</v>
       </c>
       <c r="D1" s="39" t="s">
         <v>388</v>
       </c>
       <c r="E1" s="38" t="s">
-        <v>519</v>
+        <v>540</v>
       </c>
       <c r="F1" s="3"/>
       <c r="G1" s="3"/>
@@ -14178,542 +14557,542 @@
       <c r="A2" s="8">
         <v>1</v>
       </c>
-      <c r="B2" s="54" t="s">
-        <v>520</v>
+      <c r="B2" s="58" t="s">
+        <v>541</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>521</v>
+        <v>542</v>
       </c>
       <c r="D2" s="40" t="s">
-        <v>522</v>
+        <v>543</v>
       </c>
       <c r="E2" s="40" t="s">
-        <v>523</v>
+        <v>544</v>
       </c>
     </row>
     <row r="3" spans="1:24" ht="177.75" customHeight="1">
       <c r="A3" s="8">
         <v>2</v>
       </c>
-      <c r="B3" s="54"/>
+      <c r="B3" s="58"/>
       <c r="C3" s="9" t="s">
-        <v>524</v>
+        <v>545</v>
       </c>
       <c r="D3" s="40" t="s">
-        <v>525</v>
+        <v>546</v>
       </c>
       <c r="E3" s="41" t="s">
-        <v>526</v>
+        <v>547</v>
       </c>
     </row>
     <row r="4" spans="1:24" ht="201.75">
       <c r="A4" s="8">
         <v>3</v>
       </c>
-      <c r="B4" s="54"/>
+      <c r="B4" s="58"/>
       <c r="C4" s="8" t="s">
-        <v>527</v>
+        <v>548</v>
       </c>
       <c r="D4" s="41" t="s">
-        <v>528</v>
+        <v>549</v>
       </c>
       <c r="E4" s="42" t="s">
-        <v>529</v>
+        <v>550</v>
       </c>
     </row>
     <row r="5" spans="1:24" ht="156" customHeight="1">
       <c r="A5" s="8">
         <v>4</v>
       </c>
-      <c r="B5" s="54"/>
+      <c r="B5" s="58"/>
       <c r="C5" s="8" t="s">
-        <v>530</v>
+        <v>551</v>
       </c>
       <c r="D5" s="40" t="s">
-        <v>531</v>
+        <v>552</v>
       </c>
       <c r="E5" s="40" t="s">
-        <v>532</v>
+        <v>553</v>
       </c>
     </row>
     <row r="6" spans="1:24" ht="174" customHeight="1">
       <c r="A6" s="8">
         <v>5</v>
       </c>
-      <c r="B6" s="54"/>
+      <c r="B6" s="58"/>
       <c r="C6" s="9" t="s">
-        <v>533</v>
+        <v>554</v>
       </c>
       <c r="D6" s="43" t="s">
-        <v>534</v>
+        <v>555</v>
       </c>
       <c r="E6" s="40" t="s">
-        <v>535</v>
+        <v>556</v>
       </c>
     </row>
     <row r="7" spans="1:24" ht="144.75">
       <c r="A7" s="8">
         <v>6</v>
       </c>
-      <c r="B7" s="54"/>
+      <c r="B7" s="58"/>
       <c r="C7" s="8" t="s">
-        <v>536</v>
+        <v>557</v>
       </c>
       <c r="D7" s="40" t="s">
-        <v>537</v>
+        <v>558</v>
       </c>
       <c r="E7" s="40" t="s">
-        <v>538</v>
+        <v>559</v>
       </c>
     </row>
     <row r="8" spans="1:24" ht="144.75">
       <c r="A8" s="8">
         <v>7</v>
       </c>
-      <c r="B8" s="54"/>
+      <c r="B8" s="58"/>
       <c r="C8" s="8" t="s">
-        <v>539</v>
+        <v>560</v>
       </c>
       <c r="D8" s="40" t="s">
-        <v>540</v>
+        <v>561</v>
       </c>
       <c r="E8" s="37" t="s">
-        <v>541</v>
+        <v>562</v>
       </c>
     </row>
     <row r="9" spans="1:24" ht="144.75">
       <c r="A9" s="8">
         <v>8</v>
       </c>
-      <c r="B9" s="54"/>
+      <c r="B9" s="58"/>
       <c r="C9" s="8" t="s">
-        <v>542</v>
+        <v>563</v>
       </c>
       <c r="D9" s="40" t="s">
-        <v>543</v>
+        <v>564</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>544</v>
+        <v>565</v>
       </c>
     </row>
     <row r="10" spans="1:24" ht="138.75" customHeight="1">
       <c r="A10" s="8">
         <v>9</v>
       </c>
-      <c r="B10" s="54"/>
+      <c r="B10" s="58"/>
       <c r="C10" s="8" t="s">
-        <v>545</v>
+        <v>566</v>
       </c>
       <c r="D10" s="37" t="s">
-        <v>546</v>
+        <v>567</v>
       </c>
       <c r="E10" s="37" t="s">
-        <v>547</v>
+        <v>568</v>
       </c>
     </row>
     <row r="11" spans="1:24" ht="146.25" customHeight="1">
       <c r="A11" s="8">
         <v>10</v>
       </c>
-      <c r="B11" s="54"/>
+      <c r="B11" s="58"/>
       <c r="C11" s="9" t="s">
-        <v>548</v>
+        <v>569</v>
       </c>
       <c r="D11" s="40" t="s">
-        <v>549</v>
+        <v>570</v>
       </c>
       <c r="E11" s="37" t="s">
-        <v>550</v>
+        <v>571</v>
       </c>
     </row>
     <row r="12" spans="1:24" ht="126.75" customHeight="1">
       <c r="A12" s="8">
         <v>11</v>
       </c>
-      <c r="B12" s="54"/>
+      <c r="B12" s="58"/>
       <c r="C12" s="8" t="s">
-        <v>551</v>
+        <v>572</v>
       </c>
       <c r="D12" s="40" t="s">
-        <v>552</v>
+        <v>573</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>553</v>
+        <v>574</v>
       </c>
     </row>
     <row r="13" spans="1:24" ht="144.75">
       <c r="A13" s="8">
         <v>12</v>
       </c>
-      <c r="B13" s="54"/>
+      <c r="B13" s="58"/>
       <c r="C13" s="8" t="s">
-        <v>554</v>
+        <v>575</v>
       </c>
       <c r="D13" s="40" t="s">
-        <v>555</v>
+        <v>576</v>
       </c>
       <c r="E13" s="37" t="s">
-        <v>556</v>
+        <v>577</v>
       </c>
     </row>
     <row r="14" spans="1:24" ht="115.5">
       <c r="A14" s="8">
         <v>13</v>
       </c>
-      <c r="B14" s="54"/>
+      <c r="B14" s="58"/>
       <c r="C14" s="8" t="s">
-        <v>557</v>
+        <v>578</v>
       </c>
       <c r="D14" s="40" t="s">
-        <v>558</v>
+        <v>579</v>
       </c>
       <c r="E14" s="37" t="s">
-        <v>559</v>
+        <v>580</v>
       </c>
     </row>
     <row r="15" spans="1:24" ht="115.5">
       <c r="A15" s="8">
         <v>14</v>
       </c>
-      <c r="B15" s="54"/>
+      <c r="B15" s="58"/>
       <c r="C15" s="40" t="s">
-        <v>560</v>
+        <v>581</v>
       </c>
       <c r="D15" s="37" t="s">
-        <v>561</v>
+        <v>582</v>
       </c>
       <c r="E15" s="37" t="s">
-        <v>562</v>
+        <v>583</v>
       </c>
     </row>
     <row r="16" spans="1:24" ht="144.75" customHeight="1">
       <c r="A16" s="8">
         <v>15</v>
       </c>
-      <c r="B16" s="54"/>
+      <c r="B16" s="58"/>
       <c r="C16" s="37" t="s">
-        <v>563</v>
+        <v>584</v>
       </c>
       <c r="D16" s="40" t="s">
-        <v>564</v>
+        <v>585</v>
       </c>
       <c r="E16" s="37" t="s">
-        <v>565</v>
+        <v>586</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="132" customHeight="1">
       <c r="A17" s="8">
         <v>16</v>
       </c>
-      <c r="B17" s="54"/>
+      <c r="B17" s="58"/>
       <c r="C17" s="37" t="s">
-        <v>566</v>
+        <v>587</v>
       </c>
       <c r="D17" s="37" t="s">
-        <v>567</v>
+        <v>588</v>
       </c>
       <c r="E17" s="37" t="s">
-        <v>568</v>
+        <v>589</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="115.5">
       <c r="A18" s="8">
         <v>17</v>
       </c>
-      <c r="B18" s="54"/>
+      <c r="B18" s="58"/>
       <c r="C18" s="37" t="s">
-        <v>569</v>
+        <v>590</v>
       </c>
       <c r="D18" s="37" t="s">
-        <v>570</v>
+        <v>591</v>
       </c>
       <c r="E18" s="37" t="s">
-        <v>571</v>
+        <v>592</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="115.5">
       <c r="A19" s="8">
         <v>18</v>
       </c>
-      <c r="B19" s="54"/>
+      <c r="B19" s="58"/>
       <c r="C19" s="40" t="s">
-        <v>572</v>
+        <v>593</v>
       </c>
       <c r="D19" s="40" t="s">
-        <v>573</v>
+        <v>594</v>
       </c>
       <c r="E19" s="40" t="s">
-        <v>574</v>
+        <v>595</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="87">
       <c r="A20" s="8">
         <v>19</v>
       </c>
-      <c r="B20" s="54"/>
+      <c r="B20" s="58"/>
       <c r="C20" s="37" t="s">
-        <v>575</v>
+        <v>596</v>
       </c>
       <c r="D20" s="37" t="s">
-        <v>576</v>
+        <v>597</v>
       </c>
       <c r="E20" s="37" t="s">
-        <v>577</v>
+        <v>598</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="115.5">
       <c r="A21" s="8">
         <v>20</v>
       </c>
-      <c r="B21" s="54"/>
+      <c r="B21" s="58"/>
       <c r="C21" s="37" t="s">
-        <v>578</v>
+        <v>599</v>
       </c>
       <c r="D21" s="37" t="s">
-        <v>579</v>
+        <v>600</v>
       </c>
       <c r="E21" s="37" t="s">
-        <v>580</v>
+        <v>601</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="115.5">
       <c r="A22" s="8">
         <v>21</v>
       </c>
-      <c r="B22" s="54"/>
+      <c r="B22" s="58"/>
       <c r="C22" s="44" t="s">
-        <v>581</v>
+        <v>602</v>
       </c>
       <c r="D22" s="40" t="s">
-        <v>582</v>
+        <v>603</v>
       </c>
       <c r="E22" s="37" t="s">
-        <v>583</v>
+        <v>604</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="115.5">
       <c r="A23" s="8">
         <v>22</v>
       </c>
-      <c r="B23" s="54"/>
+      <c r="B23" s="58"/>
       <c r="C23" s="40" t="s">
-        <v>584</v>
+        <v>605</v>
       </c>
       <c r="D23" s="40" t="s">
-        <v>585</v>
+        <v>606</v>
       </c>
       <c r="E23" s="37" t="s">
-        <v>586</v>
+        <v>607</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="72.75">
       <c r="A24" s="8">
         <v>23</v>
       </c>
-      <c r="B24" s="54"/>
+      <c r="B24" s="58"/>
       <c r="C24" s="40" t="s">
-        <v>587</v>
+        <v>608</v>
       </c>
       <c r="D24" s="40" t="s">
-        <v>588</v>
+        <v>609</v>
       </c>
       <c r="E24" s="40" t="s">
-        <v>587</v>
+        <v>610</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="87">
       <c r="A25" s="8">
         <v>24</v>
       </c>
-      <c r="B25" s="54"/>
+      <c r="B25" s="58"/>
       <c r="C25" s="40" t="s">
-        <v>589</v>
+        <v>611</v>
       </c>
       <c r="D25" s="40" t="s">
-        <v>590</v>
+        <v>612</v>
       </c>
       <c r="E25" s="40" t="s">
-        <v>589</v>
+        <v>613</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="72.75">
       <c r="A26" s="8">
         <v>25</v>
       </c>
-      <c r="B26" s="54"/>
+      <c r="B26" s="58"/>
       <c r="C26" s="40" t="s">
-        <v>591</v>
+        <v>614</v>
       </c>
       <c r="D26" s="40" t="s">
-        <v>592</v>
+        <v>615</v>
       </c>
       <c r="E26" s="40" t="s">
-        <v>591</v>
+        <v>616</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="87">
       <c r="A27" s="8">
         <v>26</v>
       </c>
-      <c r="B27" s="54"/>
+      <c r="B27" s="58"/>
       <c r="C27" s="40" t="s">
-        <v>593</v>
+        <v>617</v>
       </c>
       <c r="D27" s="40" t="s">
-        <v>594</v>
+        <v>618</v>
       </c>
       <c r="E27" s="40" t="s">
-        <v>593</v>
+        <v>619</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="72.75">
       <c r="A28" s="8">
         <v>27</v>
       </c>
-      <c r="B28" s="54"/>
+      <c r="B28" s="58"/>
       <c r="C28" s="8" t="s">
-        <v>595</v>
+        <v>620</v>
       </c>
       <c r="D28" s="40" t="s">
-        <v>596</v>
+        <v>621</v>
       </c>
       <c r="E28" s="45" t="s">
-        <v>595</v>
+        <v>622</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="87">
       <c r="A29" s="8">
         <v>28</v>
       </c>
-      <c r="B29" s="54"/>
+      <c r="B29" s="58"/>
       <c r="C29" s="40" t="s">
-        <v>597</v>
+        <v>623</v>
       </c>
       <c r="D29" s="40" t="s">
-        <v>598</v>
+        <v>624</v>
       </c>
       <c r="E29" s="40" t="s">
-        <v>599</v>
+        <v>625</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="72.75">
       <c r="A30" s="8">
         <v>29</v>
       </c>
-      <c r="B30" s="54"/>
+      <c r="B30" s="58"/>
       <c r="C30" s="40" t="s">
-        <v>600</v>
+        <v>626</v>
       </c>
       <c r="D30" s="40" t="s">
-        <v>601</v>
+        <v>627</v>
       </c>
       <c r="E30" s="40" t="s">
-        <v>600</v>
+        <v>628</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="72.75">
       <c r="A31" s="8">
         <v>30</v>
       </c>
-      <c r="B31" s="54"/>
+      <c r="B31" s="58"/>
       <c r="C31" s="40" t="s">
-        <v>602</v>
+        <v>629</v>
       </c>
       <c r="D31" s="40" t="s">
-        <v>603</v>
+        <v>630</v>
       </c>
       <c r="E31" s="40" t="s">
-        <v>602</v>
+        <v>631</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="72.75">
       <c r="A32" s="8">
         <v>31</v>
       </c>
-      <c r="B32" s="54"/>
+      <c r="B32" s="58"/>
       <c r="C32" s="40" t="s">
-        <v>604</v>
+        <v>632</v>
       </c>
       <c r="D32" s="40" t="s">
-        <v>605</v>
+        <v>633</v>
       </c>
       <c r="E32" s="40" t="s">
-        <v>604</v>
+        <v>634</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="57.75">
       <c r="A33" s="8">
         <v>32</v>
       </c>
-      <c r="B33" s="54"/>
+      <c r="B33" s="58"/>
       <c r="C33" s="40" t="s">
-        <v>606</v>
+        <v>635</v>
       </c>
       <c r="D33" s="40" t="s">
-        <v>607</v>
+        <v>636</v>
       </c>
       <c r="E33" s="40" t="s">
-        <v>606</v>
+        <v>637</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="57.75">
       <c r="A34" s="8">
         <v>33</v>
       </c>
-      <c r="B34" s="54"/>
+      <c r="B34" s="58"/>
       <c r="C34" s="40" t="s">
-        <v>608</v>
+        <v>638</v>
       </c>
       <c r="D34" s="40" t="s">
-        <v>609</v>
+        <v>639</v>
       </c>
       <c r="E34" s="40" t="s">
-        <v>608</v>
+        <v>640</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="57.75">
       <c r="A35" s="8">
         <v>34</v>
       </c>
-      <c r="B35" s="54"/>
+      <c r="B35" s="58"/>
       <c r="C35" s="40" t="s">
-        <v>610</v>
+        <v>641</v>
       </c>
       <c r="D35" s="40" t="s">
-        <v>611</v>
+        <v>642</v>
       </c>
       <c r="E35" s="40" t="s">
-        <v>610</v>
+        <v>643</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="57.75">
       <c r="A36" s="8">
         <v>35</v>
       </c>
-      <c r="B36" s="54"/>
+      <c r="B36" s="58"/>
       <c r="C36" s="40" t="s">
-        <v>612</v>
+        <v>644</v>
       </c>
       <c r="D36" s="40" t="s">
-        <v>613</v>
+        <v>645</v>
       </c>
       <c r="E36" s="40" t="s">
-        <v>612</v>
+        <v>646</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="87">
       <c r="A37" s="8">
         <v>36</v>
       </c>
-      <c r="B37" s="54"/>
+      <c r="B37" s="58"/>
       <c r="C37" s="8" t="s">
-        <v>614</v>
+        <v>647</v>
       </c>
       <c r="D37" s="40" t="s">
-        <v>615</v>
+        <v>648</v>
       </c>
       <c r="E37" s="8" t="s">
-        <v>614</v>
+        <v>649</v>
       </c>
     </row>
     <row r="38" spans="1:5"/>

</xml_diff>